<commit_message>
Extend values in BCpUC-energy to cover 2024
</commit_message>
<xml_diff>
--- a/InputData/elec/BCpUC/Battery Cost per Unit Cap.xlsx
+++ b/InputData/elec/BCpUC/Battery Cost per Unit Cap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BCpUC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB6724F2-1A41-4679-A919-9BC9B9ABD18B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4D004E-9358-4857-BE9A-195C5BF97CD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="839" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="839" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -1971,15 +1971,69 @@
     <xf numFmtId="5" fontId="10" fillId="14" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="169" fontId="10" fillId="14" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="59" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
@@ -2026,60 +2080,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="59" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2597,6 +2597,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2604,7 +2605,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3115,6 +3115,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3122,7 +3123,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4614,23 +4614,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.5703125" customWidth="1"/>
-    <col min="2" max="2" width="67.140625" customWidth="1"/>
+    <col min="1" max="1" width="28.54296875" customWidth="1"/>
+    <col min="2" max="2" width="67.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -4638,187 +4638,187 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" s="4">
         <v>2014</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B13" s="4">
         <v>2013</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B18" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B20" s="4">
         <v>2024</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B25" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B27" s="4">
         <v>2018</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>1.0549999999999999</v>
       </c>
@@ -4826,7 +4826,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" s="38">
         <v>0.9143273584567535</v>
       </c>
@@ -4834,7 +4834,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="38">
         <v>0.89805481563188172</v>
       </c>
@@ -4842,7 +4842,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="38">
         <v>0.88711067149387013</v>
       </c>
@@ -4850,7 +4850,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="38">
         <v>0.84730412960844359</v>
       </c>
@@ -4862,7 +4862,7 @@
         <v>0.92590251319813455</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="38">
         <v>0.78452102304761584</v>
       </c>
@@ -4870,12 +4870,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>132</v>
       </c>
@@ -4896,36 +4896,36 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{734360E0-DC8F-4FFB-9748-D4950767514E}">
   <dimension ref="A1:DD222"/>
-  <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.42578125" customWidth="1"/>
-    <col min="4" max="4" width="36.42578125" customWidth="1"/>
-    <col min="5" max="5" width="34.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.42578125" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="4.453125" customWidth="1"/>
+    <col min="4" max="4" width="36.453125" customWidth="1"/>
+    <col min="5" max="5" width="34.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.453125" customWidth="1"/>
+    <col min="7" max="7" width="12.453125" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
-    <col min="13" max="13" width="10.42578125" customWidth="1"/>
+    <col min="13" max="13" width="10.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:108" s="40" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="142" t="s">
+    <row r="1" spans="1:108" s="40" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A1" s="165" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="142"/>
-      <c r="C1" s="142"/>
-      <c r="D1" s="142"/>
-      <c r="E1" s="142"/>
-      <c r="F1" s="142"/>
-      <c r="G1" s="142"/>
-      <c r="H1" s="142"/>
-      <c r="I1" s="142"/>
-      <c r="J1" s="142"/>
-      <c r="K1" s="142"/>
+      <c r="B1" s="165"/>
+      <c r="C1" s="165"/>
+      <c r="D1" s="165"/>
+      <c r="E1" s="165"/>
+      <c r="F1" s="165"/>
+      <c r="G1" s="165"/>
+      <c r="H1" s="165"/>
+      <c r="I1" s="165"/>
+      <c r="J1" s="165"/>
+      <c r="K1" s="165"/>
       <c r="M1" s="3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2"/>
       <c r="B2"/>
       <c r="C2"/>
@@ -5037,7 +5037,7 @@
       <c r="DC2" s="41"/>
       <c r="DD2" s="41"/>
     </row>
-    <row r="3" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3"/>
       <c r="B3"/>
       <c r="C3"/>
@@ -5048,16 +5048,16 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D4" s="44"/>
-      <c r="L4" s="143" t="s">
+      <c r="L4" s="166" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:108" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="L5" s="144"/>
-    </row>
-    <row r="6" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:108" ht="14.9" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L5" s="167"/>
+    </row>
+    <row r="6" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H6" s="45"/>
       <c r="I6" s="46"/>
       <c r="J6" s="46"/>
@@ -5083,27 +5083,27 @@
       <c r="AE6" s="47"/>
       <c r="AF6" s="48"/>
     </row>
-    <row r="7" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="145" t="s">
+      <c r="C7" s="161" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="145"/>
-      <c r="E7" s="145"/>
-      <c r="F7" s="145"/>
-      <c r="G7" s="145"/>
-      <c r="H7" s="145"/>
-      <c r="I7" s="145"/>
-      <c r="J7" s="145"/>
-      <c r="K7" s="145"/>
-      <c r="L7" s="145"/>
-      <c r="M7" s="145"/>
-      <c r="N7" s="145"/>
-      <c r="O7" s="145"/>
-      <c r="P7" s="145"/>
-      <c r="Q7" s="145"/>
+      <c r="D7" s="161"/>
+      <c r="E7" s="161"/>
+      <c r="F7" s="161"/>
+      <c r="G7" s="161"/>
+      <c r="H7" s="161"/>
+      <c r="I7" s="161"/>
+      <c r="J7" s="161"/>
+      <c r="K7" s="161"/>
+      <c r="L7" s="161"/>
+      <c r="M7" s="161"/>
+      <c r="N7" s="161"/>
+      <c r="O7" s="161"/>
+      <c r="P7" s="161"/>
+      <c r="Q7" s="161"/>
       <c r="R7" s="50"/>
       <c r="S7" s="50"/>
       <c r="T7" s="50"/>
@@ -5116,67 +5116,67 @@
       <c r="AA7" s="51"/>
       <c r="AB7" s="48"/>
     </row>
-    <row r="8" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="O8" s="52"/>
     </row>
-    <row r="9" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9"/>
-      <c r="B9" s="146" t="s">
+      <c r="B9" s="168" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="147" t="s">
+      <c r="D9" s="169" t="s">
         <v>75</v>
       </c>
-      <c r="E9" s="148"/>
-      <c r="F9" s="149"/>
-      <c r="G9" s="150">
+      <c r="E9" s="170"/>
+      <c r="F9" s="171"/>
+      <c r="G9" s="172">
         <v>2022</v>
       </c>
-      <c r="H9" s="151"/>
-      <c r="I9" s="151"/>
-      <c r="J9" s="151"/>
-      <c r="K9" s="152"/>
-      <c r="L9" s="152"/>
-    </row>
-    <row r="10" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="146"/>
+      <c r="H9" s="173"/>
+      <c r="I9" s="173"/>
+      <c r="J9" s="173"/>
+      <c r="K9" s="174"/>
+      <c r="L9" s="174"/>
+    </row>
+    <row r="10" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="168"/>
       <c r="D10" s="53" t="s">
         <v>146</v>
       </c>
       <c r="J10" s="52"/>
     </row>
-    <row r="11" spans="1:108" s="40" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="146"/>
-      <c r="D11" s="153" t="s">
+    <row r="11" spans="1:108" s="40" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B11" s="168"/>
+      <c r="D11" s="175" t="s">
         <v>76</v>
       </c>
-      <c r="E11" s="154"/>
-      <c r="F11" s="154"/>
-      <c r="G11" s="154"/>
-      <c r="H11" s="154"/>
-      <c r="I11" s="154"/>
-      <c r="J11" s="154"/>
-      <c r="K11" s="154"/>
-      <c r="L11" s="154"/>
+      <c r="E11" s="176"/>
+      <c r="F11" s="176"/>
+      <c r="G11" s="176"/>
+      <c r="H11" s="176"/>
+      <c r="I11" s="176"/>
+      <c r="J11" s="176"/>
+      <c r="K11" s="176"/>
+      <c r="L11" s="176"/>
       <c r="W11" s="54"/>
       <c r="X11" s="55"/>
       <c r="Y11" s="55"/>
       <c r="Z11" s="55"/>
       <c r="AA11" s="55"/>
     </row>
-    <row r="12" spans="1:108" s="40" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="146"/>
-      <c r="D12" s="155" t="s">
+    <row r="12" spans="1:108" s="40" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="168"/>
+      <c r="D12" s="177" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="156"/>
-      <c r="F12" s="156"/>
-      <c r="G12" s="156"/>
-      <c r="H12" s="156"/>
-      <c r="I12" s="156"/>
-      <c r="J12" s="156"/>
-      <c r="K12" s="156"/>
-      <c r="L12" s="157"/>
+      <c r="E12" s="178"/>
+      <c r="F12" s="178"/>
+      <c r="G12" s="178"/>
+      <c r="H12" s="178"/>
+      <c r="I12" s="178"/>
+      <c r="J12" s="178"/>
+      <c r="K12" s="178"/>
+      <c r="L12" s="179"/>
       <c r="M12" s="56"/>
       <c r="W12" s="54"/>
       <c r="X12" s="55"/>
@@ -5184,77 +5184,77 @@
       <c r="Z12" s="55"/>
       <c r="AA12" s="55"/>
     </row>
-    <row r="13" spans="1:108" s="40" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="146"/>
-      <c r="D13" s="158"/>
-      <c r="E13" s="159"/>
-      <c r="F13" s="159"/>
-      <c r="G13" s="159"/>
-      <c r="H13" s="159"/>
-      <c r="I13" s="159"/>
-      <c r="J13" s="159"/>
-      <c r="K13" s="159"/>
-      <c r="L13" s="160"/>
+    <row r="13" spans="1:108" s="40" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B13" s="168"/>
+      <c r="D13" s="180"/>
+      <c r="E13" s="181"/>
+      <c r="F13" s="181"/>
+      <c r="G13" s="181"/>
+      <c r="H13" s="181"/>
+      <c r="I13" s="181"/>
+      <c r="J13" s="181"/>
+      <c r="K13" s="181"/>
+      <c r="L13" s="182"/>
       <c r="W13" s="54"/>
       <c r="X13" s="55"/>
       <c r="Y13" s="55"/>
       <c r="Z13" s="55"/>
       <c r="AA13" s="55"/>
     </row>
-    <row r="14" spans="1:108" ht="37.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="146"/>
-    </row>
-    <row r="15" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="146"/>
-      <c r="C15" s="161" t="s">
+    <row r="14" spans="1:108" ht="37.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="168"/>
+    </row>
+    <row r="15" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="168"/>
+      <c r="C15" s="183" t="s">
         <v>147</v>
       </c>
-      <c r="D15" s="161"/>
-      <c r="E15" s="161"/>
-      <c r="F15" s="161"/>
-      <c r="G15" s="161"/>
-      <c r="H15" s="161"/>
-      <c r="I15" s="161"/>
-      <c r="J15" s="161"/>
-      <c r="K15" s="161"/>
-      <c r="L15" s="161"/>
-      <c r="M15" s="161"/>
-      <c r="N15" s="161"/>
-      <c r="O15" s="161"/>
-      <c r="P15" s="161"/>
+      <c r="D15" s="183"/>
+      <c r="E15" s="183"/>
+      <c r="F15" s="183"/>
+      <c r="G15" s="183"/>
+      <c r="H15" s="183"/>
+      <c r="I15" s="183"/>
+      <c r="J15" s="183"/>
+      <c r="K15" s="183"/>
+      <c r="L15" s="183"/>
+      <c r="M15" s="183"/>
+      <c r="N15" s="183"/>
+      <c r="O15" s="183"/>
+      <c r="P15" s="183"/>
       <c r="Q15" s="57"/>
     </row>
-    <row r="16" spans="1:108" x14ac:dyDescent="0.25">
-      <c r="B16" s="146"/>
-      <c r="C16" s="161"/>
-      <c r="D16" s="161"/>
-      <c r="E16" s="161"/>
-      <c r="F16" s="161"/>
-      <c r="G16" s="161"/>
-      <c r="H16" s="161"/>
-      <c r="I16" s="161"/>
-      <c r="J16" s="161"/>
-      <c r="K16" s="161"/>
-      <c r="L16" s="161"/>
-      <c r="M16" s="161"/>
-      <c r="N16" s="161"/>
-      <c r="O16" s="161"/>
-      <c r="P16" s="161"/>
-    </row>
-    <row r="17" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="146"/>
+    <row r="16" spans="1:108" x14ac:dyDescent="0.35">
+      <c r="B16" s="168"/>
+      <c r="C16" s="183"/>
+      <c r="D16" s="183"/>
+      <c r="E16" s="183"/>
+      <c r="F16" s="183"/>
+      <c r="G16" s="183"/>
+      <c r="H16" s="183"/>
+      <c r="I16" s="183"/>
+      <c r="J16" s="183"/>
+      <c r="K16" s="183"/>
+      <c r="L16" s="183"/>
+      <c r="M16" s="183"/>
+      <c r="N16" s="183"/>
+      <c r="O16" s="183"/>
+      <c r="P16" s="183"/>
+    </row>
+    <row r="17" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="168"/>
       <c r="C17" s="58"/>
-      <c r="D17" s="168" t="s">
+      <c r="D17" s="158" t="s">
         <v>78</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="18" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="146"/>
+    <row r="18" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="168"/>
       <c r="C18" s="58"/>
-      <c r="D18" s="169"/>
+      <c r="D18" s="159"/>
       <c r="F18" s="1" t="s">
         <v>145</v>
       </c>
@@ -5346,10 +5346,10 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="19" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="146"/>
+    <row r="19" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="168"/>
       <c r="C19" s="58"/>
-      <c r="D19" s="169"/>
+      <c r="D19" s="159"/>
       <c r="E19" t="s">
         <v>80</v>
       </c>
@@ -5444,10 +5444,10 @@
         <v>129.15171555556242</v>
       </c>
     </row>
-    <row r="20" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="146"/>
+    <row r="20" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="168"/>
       <c r="C20" s="58"/>
-      <c r="D20" s="170"/>
+      <c r="D20" s="160"/>
       <c r="E20" t="s">
         <v>81</v>
       </c>
@@ -5542,10 +5542,10 @@
         <v>157.23705301149212</v>
       </c>
     </row>
-    <row r="21" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="146"/>
+    <row r="21" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="168"/>
       <c r="C21" s="58"/>
-      <c r="D21" s="170"/>
+      <c r="D21" s="160"/>
       <c r="E21" t="s">
         <v>82</v>
       </c>
@@ -5640,10 +5640,10 @@
         <v>274.95897351378562</v>
       </c>
     </row>
-    <row r="22" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="146"/>
+    <row r="22" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="168"/>
       <c r="C22" s="58"/>
-      <c r="D22" s="170"/>
+      <c r="D22" s="160"/>
       <c r="F22" s="60"/>
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
@@ -5675,19 +5675,19 @@
       <c r="AH22" s="5"/>
       <c r="AI22" s="5"/>
     </row>
-    <row r="23" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="146"/>
+    <row r="23" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="168"/>
       <c r="C23" s="58"/>
-      <c r="D23" s="170"/>
+      <c r="D23" s="160"/>
       <c r="E23" s="1" t="s">
         <v>83</v>
       </c>
       <c r="F23" s="60"/>
     </row>
-    <row r="24" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="146"/>
+    <row r="24" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="168"/>
       <c r="C24" s="58"/>
-      <c r="D24" s="170"/>
+      <c r="D24" s="160"/>
       <c r="F24" s="1" t="s">
         <v>145</v>
       </c>
@@ -5779,10 +5779,10 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="25" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="146"/>
+    <row r="25" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="168"/>
       <c r="C25" s="58"/>
-      <c r="D25" s="170"/>
+      <c r="D25" s="160"/>
       <c r="E25" t="s">
         <v>80</v>
       </c>
@@ -5877,10 +5877,10 @@
         <v>118.54336408357527</v>
       </c>
     </row>
-    <row r="26" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="146"/>
+    <row r="26" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B26" s="168"/>
       <c r="C26" s="58"/>
-      <c r="D26" s="170"/>
+      <c r="D26" s="160"/>
       <c r="E26" t="s">
         <v>81</v>
       </c>
@@ -5975,10 +5975,10 @@
         <v>270.30971238933148</v>
       </c>
     </row>
-    <row r="27" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="146"/>
+    <row r="27" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B27" s="168"/>
       <c r="C27" s="58"/>
-      <c r="D27" s="170"/>
+      <c r="D27" s="160"/>
       <c r="E27" t="s">
         <v>82</v>
       </c>
@@ -6073,8 +6073,8 @@
         <v>291.72086922260991</v>
       </c>
     </row>
-    <row r="28" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="146"/>
+    <row r="28" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="168"/>
       <c r="C28" s="58"/>
       <c r="D28" s="58"/>
       <c r="G28" s="5"/>
@@ -6111,8 +6111,8 @@
       <c r="AL28" s="5"/>
       <c r="AM28" s="5"/>
     </row>
-    <row r="29" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="146"/>
+    <row r="29" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="168"/>
       <c r="C29" s="58"/>
       <c r="D29" s="58"/>
       <c r="E29" s="1" t="s">
@@ -6153,8 +6153,8 @@
       <c r="AL29" s="5"/>
       <c r="AM29" s="5"/>
     </row>
-    <row r="30" spans="2:39" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="146"/>
+    <row r="30" spans="2:39" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B30" s="168"/>
       <c r="C30" s="58"/>
       <c r="D30" s="58"/>
       <c r="E30" s="1"/>
@@ -6193,10 +6193,10 @@
       <c r="AL30" s="5"/>
       <c r="AM30" s="5"/>
     </row>
-    <row r="31" spans="2:39" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="146"/>
+    <row r="31" spans="2:39" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B31" s="168"/>
       <c r="C31" s="58"/>
-      <c r="D31" s="169" t="s">
+      <c r="D31" s="159" t="s">
         <v>85</v>
       </c>
       <c r="E31" s="61" t="s">
@@ -6245,10 +6245,10 @@
       <c r="AL31" s="5"/>
       <c r="AM31" s="5"/>
     </row>
-    <row r="32" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="146"/>
+    <row r="32" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="168"/>
       <c r="C32" s="58"/>
-      <c r="D32" s="169"/>
+      <c r="D32" s="159"/>
       <c r="E32" s="66" t="s">
         <v>91</v>
       </c>
@@ -6295,10 +6295,10 @@
       <c r="AL32" s="5"/>
       <c r="AM32" s="5"/>
     </row>
-    <row r="33" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="146"/>
+    <row r="33" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="168"/>
       <c r="C33" s="58"/>
-      <c r="D33" s="169"/>
+      <c r="D33" s="159"/>
       <c r="E33" s="69" t="s">
         <v>96</v>
       </c>
@@ -6345,10 +6345,10 @@
       <c r="AL33" s="5"/>
       <c r="AM33" s="5"/>
     </row>
-    <row r="34" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="146"/>
+    <row r="34" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="168"/>
       <c r="C34" s="58"/>
-      <c r="D34" s="169"/>
+      <c r="D34" s="159"/>
       <c r="E34" s="72" t="s">
         <v>98</v>
       </c>
@@ -6395,10 +6395,10 @@
       <c r="AL34" s="5"/>
       <c r="AM34" s="5"/>
     </row>
-    <row r="35" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="146"/>
+    <row r="35" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B35" s="168"/>
       <c r="C35" s="58"/>
-      <c r="D35" s="169"/>
+      <c r="D35" s="159"/>
       <c r="E35" s="69" t="s">
         <v>100</v>
       </c>
@@ -6445,10 +6445,10 @@
       <c r="AL35" s="5"/>
       <c r="AM35" s="5"/>
     </row>
-    <row r="36" spans="2:74" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="146"/>
+    <row r="36" spans="2:74" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B36" s="168"/>
       <c r="C36" s="58"/>
-      <c r="D36" s="169"/>
+      <c r="D36" s="159"/>
       <c r="E36" s="75" t="s">
         <v>102</v>
       </c>
@@ -6495,7 +6495,7 @@
       <c r="AL36" s="5"/>
       <c r="AM36" s="5"/>
     </row>
-    <row r="37" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C37" s="58"/>
       <c r="D37" s="58"/>
       <c r="E37" s="1"/>
@@ -6534,24 +6534,24 @@
       <c r="AL37" s="5"/>
       <c r="AM37" s="5"/>
     </row>
-    <row r="38" spans="2:74" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C38" s="145" t="s">
+    <row r="38" spans="2:74" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C38" s="161" t="s">
         <v>104</v>
       </c>
-      <c r="D38" s="145"/>
-      <c r="E38" s="145"/>
-      <c r="F38" s="145"/>
-      <c r="G38" s="145"/>
-      <c r="H38" s="145"/>
-      <c r="I38" s="145"/>
-      <c r="J38" s="145"/>
-      <c r="K38" s="145"/>
-      <c r="L38" s="145"/>
-      <c r="M38" s="145"/>
-      <c r="N38" s="145"/>
-      <c r="O38" s="145"/>
-      <c r="P38" s="145"/>
-      <c r="Q38" s="145"/>
+      <c r="D38" s="161"/>
+      <c r="E38" s="161"/>
+      <c r="F38" s="161"/>
+      <c r="G38" s="161"/>
+      <c r="H38" s="161"/>
+      <c r="I38" s="161"/>
+      <c r="J38" s="161"/>
+      <c r="K38" s="161"/>
+      <c r="L38" s="161"/>
+      <c r="M38" s="161"/>
+      <c r="N38" s="161"/>
+      <c r="O38" s="161"/>
+      <c r="P38" s="161"/>
+      <c r="Q38" s="161"/>
       <c r="R38" s="50"/>
       <c r="S38" s="50"/>
       <c r="T38" s="50"/>
@@ -6580,18 +6580,18 @@
       <c r="AQ38" s="78"/>
       <c r="AR38" s="78"/>
     </row>
-    <row r="39" spans="2:74" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="2:74" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:74" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="2:74" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D40" s="53" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="41" spans="2:74" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:74" x14ac:dyDescent="0.35">
       <c r="D41" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="2:74" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:74" x14ac:dyDescent="0.35">
       <c r="G42" s="1" t="s">
         <v>145</v>
       </c>
@@ -6683,11 +6683,11 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="43" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="177" t="s">
+    <row r="43" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B43" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="D43" s="168" t="s">
+      <c r="D43" s="158" t="s">
         <v>106</v>
       </c>
       <c r="E43" s="79" t="s">
@@ -6788,9 +6788,9 @@
         <v>376.84679519470012</v>
       </c>
     </row>
-    <row r="44" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B44" s="177"/>
-      <c r="D44" s="169"/>
+    <row r="44" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B44" s="163"/>
+      <c r="D44" s="159"/>
       <c r="E44" s="82" t="s">
         <v>91</v>
       </c>
@@ -6889,9 +6889,9 @@
         <v>584.78381841231567</v>
       </c>
     </row>
-    <row r="45" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B45" s="177"/>
-      <c r="D45" s="169"/>
+    <row r="45" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B45" s="163"/>
+      <c r="D45" s="159"/>
       <c r="E45" s="83" t="s">
         <v>91</v>
       </c>
@@ -6990,9 +6990,9 @@
         <v>841.63881625018121</v>
       </c>
     </row>
-    <row r="46" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B46" s="177"/>
-      <c r="D46" s="170"/>
+    <row r="46" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B46" s="163"/>
+      <c r="D46" s="160"/>
       <c r="E46" s="79" t="s">
         <v>96</v>
       </c>
@@ -7124,9 +7124,9 @@
       <c r="BU46" s="5"/>
       <c r="BV46" s="5"/>
     </row>
-    <row r="47" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B47" s="177"/>
-      <c r="D47" s="170"/>
+    <row r="47" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B47" s="163"/>
+      <c r="D47" s="160"/>
       <c r="E47" s="79" t="s">
         <v>96</v>
       </c>
@@ -7258,9 +7258,9 @@
       <c r="BU47" s="5"/>
       <c r="BV47" s="5"/>
     </row>
-    <row r="48" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B48" s="177"/>
-      <c r="D48" s="170"/>
+    <row r="48" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B48" s="163"/>
+      <c r="D48" s="160"/>
       <c r="E48" s="79" t="s">
         <v>96</v>
       </c>
@@ -7392,9 +7392,9 @@
       <c r="BU48" s="5"/>
       <c r="BV48" s="5"/>
     </row>
-    <row r="49" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B49" s="177"/>
-      <c r="D49" s="170"/>
+    <row r="49" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B49" s="163"/>
+      <c r="D49" s="160"/>
       <c r="E49" s="79" t="s">
         <v>98</v>
       </c>
@@ -7526,9 +7526,9 @@
       <c r="BU49" s="5"/>
       <c r="BV49" s="5"/>
     </row>
-    <row r="50" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B50" s="177"/>
-      <c r="D50" s="170"/>
+    <row r="50" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B50" s="163"/>
+      <c r="D50" s="160"/>
       <c r="E50" s="79" t="s">
         <v>98</v>
       </c>
@@ -7660,9 +7660,9 @@
       <c r="BU50" s="5"/>
       <c r="BV50" s="5"/>
     </row>
-    <row r="51" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B51" s="177"/>
-      <c r="D51" s="170"/>
+    <row r="51" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B51" s="163"/>
+      <c r="D51" s="160"/>
       <c r="E51" s="79" t="s">
         <v>98</v>
       </c>
@@ -7794,9 +7794,9 @@
       <c r="BU51" s="5"/>
       <c r="BV51" s="5"/>
     </row>
-    <row r="52" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B52" s="177"/>
-      <c r="D52" s="170"/>
+    <row r="52" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B52" s="163"/>
+      <c r="D52" s="160"/>
       <c r="E52" s="79" t="s">
         <v>100</v>
       </c>
@@ -7928,9 +7928,9 @@
       <c r="BU52" s="5"/>
       <c r="BV52" s="5"/>
     </row>
-    <row r="53" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B53" s="177"/>
-      <c r="D53" s="170"/>
+    <row r="53" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B53" s="163"/>
+      <c r="D53" s="160"/>
       <c r="E53" s="79" t="s">
         <v>100</v>
       </c>
@@ -8062,9 +8062,9 @@
       <c r="BU53" s="5"/>
       <c r="BV53" s="5"/>
     </row>
-    <row r="54" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B54" s="177"/>
-      <c r="D54" s="170"/>
+    <row r="54" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B54" s="163"/>
+      <c r="D54" s="160"/>
       <c r="E54" s="79" t="s">
         <v>100</v>
       </c>
@@ -8196,9 +8196,9 @@
       <c r="BU54" s="5"/>
       <c r="BV54" s="5"/>
     </row>
-    <row r="55" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B55" s="177"/>
-      <c r="D55" s="170"/>
+    <row r="55" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B55" s="163"/>
+      <c r="D55" s="160"/>
       <c r="E55" s="79" t="s">
         <v>102</v>
       </c>
@@ -8330,9 +8330,9 @@
       <c r="BU55" s="5"/>
       <c r="BV55" s="5"/>
     </row>
-    <row r="56" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B56" s="177"/>
-      <c r="D56" s="170"/>
+    <row r="56" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B56" s="163"/>
+      <c r="D56" s="160"/>
       <c r="E56" s="79" t="s">
         <v>102</v>
       </c>
@@ -8464,9 +8464,9 @@
       <c r="BU56" s="5"/>
       <c r="BV56" s="5"/>
     </row>
-    <row r="57" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B57" s="177"/>
-      <c r="D57" s="170"/>
+    <row r="57" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B57" s="163"/>
+      <c r="D57" s="160"/>
       <c r="E57" s="79" t="s">
         <v>102</v>
       </c>
@@ -8598,8 +8598,8 @@
       <c r="BU57" s="5"/>
       <c r="BV57" s="5"/>
     </row>
-    <row r="58" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B58" s="177"/>
+    <row r="58" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B58" s="163"/>
       <c r="D58" s="58"/>
       <c r="E58" s="82"/>
       <c r="F58" s="82"/>
@@ -8667,8 +8667,8 @@
       <c r="BU58" s="5"/>
       <c r="BV58" s="5"/>
     </row>
-    <row r="59" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B59" s="177"/>
+    <row r="59" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B59" s="163"/>
       <c r="D59" s="58"/>
       <c r="E59" s="82"/>
       <c r="F59" s="82"/>
@@ -8736,8 +8736,8 @@
       <c r="BU59" s="5"/>
       <c r="BV59" s="5"/>
     </row>
-    <row r="60" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B60" s="177"/>
+    <row r="60" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B60" s="163"/>
       <c r="D60" s="58"/>
       <c r="E60" s="82"/>
       <c r="F60" s="82"/>
@@ -8805,8 +8805,8 @@
       <c r="BU60" s="5"/>
       <c r="BV60" s="5"/>
     </row>
-    <row r="61" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B61" s="177"/>
+    <row r="61" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B61" s="163"/>
       <c r="D61" s="84"/>
       <c r="E61" s="82"/>
       <c r="F61" s="82"/>
@@ -8901,9 +8901,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="62" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B62" s="177"/>
-      <c r="D62" s="168" t="s">
+    <row r="62" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B62" s="163"/>
+      <c r="D62" s="158" t="s">
         <v>107</v>
       </c>
       <c r="E62" s="79" t="s">
@@ -9004,9 +9004,9 @@
         <v>9.4211698798675041</v>
       </c>
     </row>
-    <row r="63" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B63" s="177"/>
-      <c r="D63" s="169"/>
+    <row r="63" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B63" s="163"/>
+      <c r="D63" s="159"/>
       <c r="E63" s="82" t="s">
         <v>91</v>
       </c>
@@ -9105,9 +9105,9 @@
         <v>14.619595460307892</v>
       </c>
     </row>
-    <row r="64" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B64" s="177"/>
-      <c r="D64" s="169"/>
+    <row r="64" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B64" s="163"/>
+      <c r="D64" s="159"/>
       <c r="E64" s="83" t="s">
         <v>91</v>
       </c>
@@ -9206,9 +9206,9 @@
         <v>21.04097040625453</v>
       </c>
     </row>
-    <row r="65" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B65" s="177"/>
-      <c r="D65" s="170"/>
+    <row r="65" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B65" s="163"/>
+      <c r="D65" s="160"/>
       <c r="E65" s="79" t="s">
         <v>96</v>
       </c>
@@ -9307,9 +9307,9 @@
         <v>15.878755657645625</v>
       </c>
     </row>
-    <row r="66" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B66" s="177"/>
-      <c r="D66" s="170"/>
+    <row r="66" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B66" s="163"/>
+      <c r="D66" s="160"/>
       <c r="E66" s="79" t="s">
         <v>96</v>
       </c>
@@ -9408,9 +9408,9 @@
         <v>22.4814481108825</v>
       </c>
     </row>
-    <row r="67" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B67" s="177"/>
-      <c r="D67" s="170"/>
+    <row r="67" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B67" s="163"/>
+      <c r="D67" s="160"/>
       <c r="E67" s="79" t="s">
         <v>96</v>
       </c>
@@ -9509,9 +9509,9 @@
         <v>34.78891908194381</v>
       </c>
     </row>
-    <row r="68" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B68" s="177"/>
-      <c r="D68" s="170"/>
+    <row r="68" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B68" s="163"/>
+      <c r="D68" s="160"/>
       <c r="E68" s="79" t="s">
         <v>98</v>
       </c>
@@ -9610,9 +9610,9 @@
         <v>22.336341435423748</v>
       </c>
     </row>
-    <row r="69" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B69" s="177"/>
-      <c r="D69" s="170"/>
+    <row r="69" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B69" s="163"/>
+      <c r="D69" s="160"/>
       <c r="E69" s="79" t="s">
         <v>98</v>
       </c>
@@ -9711,9 +9711,9 @@
         <v>30.343300761457108</v>
       </c>
     </row>
-    <row r="70" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B70" s="177"/>
-      <c r="D70" s="170"/>
+    <row r="70" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B70" s="163"/>
+      <c r="D70" s="160"/>
       <c r="E70" s="79" t="s">
         <v>98</v>
       </c>
@@ -9812,9 +9812,9 @@
         <v>48.536867757633097</v>
       </c>
     </row>
-    <row r="71" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B71" s="177"/>
-      <c r="D71" s="170"/>
+    <row r="71" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B71" s="163"/>
+      <c r="D71" s="160"/>
       <c r="E71" s="79" t="s">
         <v>100</v>
       </c>
@@ -9946,9 +9946,9 @@
       <c r="BU71" s="5"/>
       <c r="BV71" s="5"/>
     </row>
-    <row r="72" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B72" s="177"/>
-      <c r="D72" s="170"/>
+    <row r="72" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B72" s="163"/>
+      <c r="D72" s="160"/>
       <c r="E72" s="79" t="s">
         <v>100</v>
       </c>
@@ -10080,9 +10080,9 @@
       <c r="BU72" s="5"/>
       <c r="BV72" s="5"/>
     </row>
-    <row r="73" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B73" s="177"/>
-      <c r="D73" s="170"/>
+    <row r="73" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B73" s="163"/>
+      <c r="D73" s="160"/>
       <c r="E73" s="79" t="s">
         <v>100</v>
       </c>
@@ -10214,9 +10214,9 @@
       <c r="BU73" s="5"/>
       <c r="BV73" s="5"/>
     </row>
-    <row r="74" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B74" s="177"/>
-      <c r="D74" s="170"/>
+    <row r="74" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B74" s="163"/>
+      <c r="D74" s="160"/>
       <c r="E74" s="79" t="s">
         <v>102</v>
       </c>
@@ -10348,9 +10348,9 @@
       <c r="BU74" s="5"/>
       <c r="BV74" s="5"/>
     </row>
-    <row r="75" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B75" s="177"/>
-      <c r="D75" s="170"/>
+    <row r="75" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B75" s="163"/>
+      <c r="D75" s="160"/>
       <c r="E75" s="79" t="s">
         <v>102</v>
       </c>
@@ -10482,9 +10482,9 @@
       <c r="BU75" s="5"/>
       <c r="BV75" s="5"/>
     </row>
-    <row r="76" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B76" s="177"/>
-      <c r="D76" s="170"/>
+    <row r="76" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B76" s="163"/>
+      <c r="D76" s="160"/>
       <c r="E76" s="79" t="s">
         <v>102</v>
       </c>
@@ -10616,14 +10616,14 @@
       <c r="BU76" s="5"/>
       <c r="BV76" s="5"/>
     </row>
-    <row r="77" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B77" s="177"/>
+    <row r="77" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B77" s="163"/>
       <c r="D77" s="84"/>
       <c r="E77" s="82"/>
       <c r="F77" s="82"/>
     </row>
-    <row r="78" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B78" s="177"/>
+    <row r="78" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B78" s="163"/>
       <c r="D78" s="40"/>
       <c r="E78" s="85"/>
       <c r="F78" s="85"/>
@@ -10718,9 +10718,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="79" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B79" s="177"/>
-      <c r="D79" s="168" t="s">
+    <row r="79" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B79" s="163"/>
+      <c r="D79" s="158" t="s">
         <v>108</v>
       </c>
       <c r="E79" s="79" t="s">
@@ -10821,9 +10821,9 @@
       </c>
       <c r="AO79" s="1"/>
     </row>
-    <row r="80" spans="2:74" x14ac:dyDescent="0.25">
-      <c r="B80" s="177"/>
-      <c r="D80" s="169"/>
+    <row r="80" spans="2:74" x14ac:dyDescent="0.35">
+      <c r="B80" s="163"/>
+      <c r="D80" s="159"/>
       <c r="E80" s="82" t="s">
         <v>91</v>
       </c>
@@ -10922,9 +10922,9 @@
       </c>
       <c r="AO80" s="1"/>
     </row>
-    <row r="81" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B81" s="177"/>
-      <c r="D81" s="169"/>
+    <row r="81" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B81" s="163"/>
+      <c r="D81" s="159"/>
       <c r="E81" s="83" t="s">
         <v>91</v>
       </c>
@@ -11023,9 +11023,9 @@
       </c>
       <c r="AO81" s="1"/>
     </row>
-    <row r="82" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B82" s="178"/>
-      <c r="D82" s="170"/>
+    <row r="82" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B82" s="164"/>
+      <c r="D82" s="160"/>
       <c r="E82" s="79" t="s">
         <v>96</v>
       </c>
@@ -11123,9 +11123,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B83" s="178"/>
-      <c r="D83" s="170"/>
+    <row r="83" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B83" s="164"/>
+      <c r="D83" s="160"/>
       <c r="E83" s="79" t="s">
         <v>96</v>
       </c>
@@ -11223,9 +11223,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B84" s="178"/>
-      <c r="D84" s="170"/>
+    <row r="84" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B84" s="164"/>
+      <c r="D84" s="160"/>
       <c r="E84" s="79" t="s">
         <v>96</v>
       </c>
@@ -11325,9 +11325,9 @@
       <c r="AK84" s="5"/>
       <c r="AL84" s="5"/>
     </row>
-    <row r="85" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B85" s="178"/>
-      <c r="D85" s="170"/>
+    <row r="85" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B85" s="164"/>
+      <c r="D85" s="160"/>
       <c r="E85" s="79" t="s">
         <v>98</v>
       </c>
@@ -11427,9 +11427,9 @@
       <c r="AK85" s="5"/>
       <c r="AL85" s="5"/>
     </row>
-    <row r="86" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B86" s="178"/>
-      <c r="D86" s="170"/>
+    <row r="86" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B86" s="164"/>
+      <c r="D86" s="160"/>
       <c r="E86" s="79" t="s">
         <v>98</v>
       </c>
@@ -11529,9 +11529,9 @@
       <c r="AK86" s="5"/>
       <c r="AL86" s="5"/>
     </row>
-    <row r="87" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B87" s="178"/>
-      <c r="D87" s="170"/>
+    <row r="87" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B87" s="164"/>
+      <c r="D87" s="160"/>
       <c r="E87" s="79" t="s">
         <v>98</v>
       </c>
@@ -11631,9 +11631,9 @@
       <c r="AK87" s="5"/>
       <c r="AL87" s="5"/>
     </row>
-    <row r="88" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B88" s="178"/>
-      <c r="D88" s="170"/>
+    <row r="88" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B88" s="164"/>
+      <c r="D88" s="160"/>
       <c r="E88" s="79" t="s">
         <v>100</v>
       </c>
@@ -11733,9 +11733,9 @@
       <c r="AK88" s="5"/>
       <c r="AL88" s="5"/>
     </row>
-    <row r="89" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B89" s="178"/>
-      <c r="D89" s="170"/>
+    <row r="89" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B89" s="164"/>
+      <c r="D89" s="160"/>
       <c r="E89" s="79" t="s">
         <v>100</v>
       </c>
@@ -11835,9 +11835,9 @@
       <c r="AK89" s="5"/>
       <c r="AL89" s="5"/>
     </row>
-    <row r="90" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B90" s="178"/>
-      <c r="D90" s="170"/>
+    <row r="90" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B90" s="164"/>
+      <c r="D90" s="160"/>
       <c r="E90" s="79" t="s">
         <v>100</v>
       </c>
@@ -11937,9 +11937,9 @@
       <c r="AK90" s="5"/>
       <c r="AL90" s="5"/>
     </row>
-    <row r="91" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B91" s="178"/>
-      <c r="D91" s="170"/>
+    <row r="91" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B91" s="164"/>
+      <c r="D91" s="160"/>
       <c r="E91" s="79" t="s">
         <v>102</v>
       </c>
@@ -12039,9 +12039,9 @@
       <c r="AK91" s="5"/>
       <c r="AL91" s="5"/>
     </row>
-    <row r="92" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B92" s="178"/>
-      <c r="D92" s="170"/>
+    <row r="92" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B92" s="164"/>
+      <c r="D92" s="160"/>
       <c r="E92" s="79" t="s">
         <v>102</v>
       </c>
@@ -12141,9 +12141,9 @@
       <c r="AK92" s="5"/>
       <c r="AL92" s="5"/>
     </row>
-    <row r="93" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B93" s="178"/>
-      <c r="D93" s="170"/>
+    <row r="93" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B93" s="164"/>
+      <c r="D93" s="160"/>
       <c r="E93" s="79" t="s">
         <v>102</v>
       </c>
@@ -12243,11 +12243,11 @@
       <c r="AK93" s="5"/>
       <c r="AL93" s="5"/>
     </row>
-    <row r="94" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B94" s="178"/>
-    </row>
-    <row r="95" spans="2:41" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B95" s="178"/>
+    <row r="94" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B94" s="164"/>
+    </row>
+    <row r="95" spans="2:41" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B95" s="164"/>
       <c r="G95" s="1" t="s">
         <v>145</v>
       </c>
@@ -12339,9 +12339,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="96" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B96" s="178"/>
-      <c r="D96" s="168" t="s">
+    <row r="96" spans="2:41" x14ac:dyDescent="0.35">
+      <c r="B96" s="164"/>
+      <c r="D96" s="158" t="s">
         <v>109</v>
       </c>
       <c r="E96" s="79" t="s">
@@ -12441,9 +12441,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="97" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B97" s="178"/>
-      <c r="D97" s="169"/>
+    <row r="97" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B97" s="164"/>
+      <c r="D97" s="159"/>
       <c r="E97" s="82" t="s">
         <v>91</v>
       </c>
@@ -12541,9 +12541,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="98" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B98" s="178"/>
-      <c r="D98" s="169"/>
+    <row r="98" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B98" s="164"/>
+      <c r="D98" s="159"/>
       <c r="E98" s="83" t="s">
         <v>91</v>
       </c>
@@ -12641,9 +12641,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="99" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B99" s="178"/>
-      <c r="D99" s="170"/>
+    <row r="99" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B99" s="164"/>
+      <c r="D99" s="160"/>
       <c r="E99" s="79" t="s">
         <v>96</v>
       </c>
@@ -12741,9 +12741,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="100" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B100" s="178"/>
-      <c r="D100" s="170"/>
+    <row r="100" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B100" s="164"/>
+      <c r="D100" s="160"/>
       <c r="E100" s="79" t="s">
         <v>96</v>
       </c>
@@ -12841,9 +12841,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="101" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B101" s="178"/>
-      <c r="D101" s="170"/>
+    <row r="101" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B101" s="164"/>
+      <c r="D101" s="160"/>
       <c r="E101" s="79" t="s">
         <v>96</v>
       </c>
@@ -12941,9 +12941,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="102" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B102" s="178"/>
-      <c r="D102" s="170"/>
+    <row r="102" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B102" s="164"/>
+      <c r="D102" s="160"/>
       <c r="E102" s="79" t="s">
         <v>98</v>
       </c>
@@ -13041,9 +13041,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="103" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B103" s="178"/>
-      <c r="D103" s="170"/>
+    <row r="103" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B103" s="164"/>
+      <c r="D103" s="160"/>
       <c r="E103" s="79" t="s">
         <v>98</v>
       </c>
@@ -13141,9 +13141,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="104" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B104" s="178"/>
-      <c r="D104" s="170"/>
+    <row r="104" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B104" s="164"/>
+      <c r="D104" s="160"/>
       <c r="E104" s="79" t="s">
         <v>98</v>
       </c>
@@ -13241,9 +13241,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="105" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B105" s="178"/>
-      <c r="D105" s="170"/>
+    <row r="105" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B105" s="164"/>
+      <c r="D105" s="160"/>
       <c r="E105" s="79" t="s">
         <v>100</v>
       </c>
@@ -13341,9 +13341,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="106" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B106" s="178"/>
-      <c r="D106" s="170"/>
+    <row r="106" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B106" s="164"/>
+      <c r="D106" s="160"/>
       <c r="E106" s="79" t="s">
         <v>100</v>
       </c>
@@ -13441,9 +13441,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="107" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B107" s="178"/>
-      <c r="D107" s="170"/>
+    <row r="107" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B107" s="164"/>
+      <c r="D107" s="160"/>
       <c r="E107" s="79" t="s">
         <v>100</v>
       </c>
@@ -13541,9 +13541,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="108" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B108" s="178"/>
-      <c r="D108" s="170"/>
+    <row r="108" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B108" s="164"/>
+      <c r="D108" s="160"/>
       <c r="E108" s="79" t="s">
         <v>102</v>
       </c>
@@ -13641,9 +13641,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="109" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B109" s="178"/>
-      <c r="D109" s="170"/>
+    <row r="109" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B109" s="164"/>
+      <c r="D109" s="160"/>
       <c r="E109" s="79" t="s">
         <v>102</v>
       </c>
@@ -13741,9 +13741,9 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="110" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B110" s="178"/>
-      <c r="D110" s="170"/>
+    <row r="110" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B110" s="164"/>
+      <c r="D110" s="160"/>
       <c r="E110" s="79" t="s">
         <v>102</v>
       </c>
@@ -13841,11 +13841,11 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="111" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B111" s="178"/>
-    </row>
-    <row r="112" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B112" s="178"/>
+    <row r="111" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B111" s="164"/>
+    </row>
+    <row r="112" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B112" s="164"/>
       <c r="G112" s="1" t="s">
         <v>145</v>
       </c>
@@ -13937,9 +13937,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="113" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B113" s="178"/>
-      <c r="D113" s="168" t="s">
+    <row r="113" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B113" s="164"/>
+      <c r="D113" s="158" t="s">
         <v>110</v>
       </c>
       <c r="E113" s="79" t="s">
@@ -14040,9 +14040,9 @@
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="114" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B114" s="178"/>
-      <c r="D114" s="169"/>
+    <row r="114" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B114" s="164"/>
+      <c r="D114" s="159"/>
       <c r="E114" s="82" t="s">
         <v>91</v>
       </c>
@@ -14141,9 +14141,9 @@
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="115" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B115" s="178"/>
-      <c r="D115" s="169"/>
+    <row r="115" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B115" s="164"/>
+      <c r="D115" s="159"/>
       <c r="E115" s="83" t="s">
         <v>91</v>
       </c>
@@ -14242,9 +14242,9 @@
         <v>8.3333333333333329E-2</v>
       </c>
     </row>
-    <row r="116" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B116" s="178"/>
-      <c r="D116" s="170"/>
+    <row r="116" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B116" s="164"/>
+      <c r="D116" s="160"/>
       <c r="E116" s="79" t="s">
         <v>96</v>
       </c>
@@ -14343,9 +14343,9 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="117" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B117" s="178"/>
-      <c r="D117" s="170"/>
+    <row r="117" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B117" s="164"/>
+      <c r="D117" s="160"/>
       <c r="E117" s="79" t="s">
         <v>96</v>
       </c>
@@ -14444,9 +14444,9 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="118" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B118" s="178"/>
-      <c r="D118" s="170"/>
+    <row r="118" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B118" s="164"/>
+      <c r="D118" s="160"/>
       <c r="E118" s="79" t="s">
         <v>96</v>
       </c>
@@ -14545,9 +14545,9 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="119" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B119" s="178"/>
-      <c r="D119" s="170"/>
+    <row r="119" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B119" s="164"/>
+      <c r="D119" s="160"/>
       <c r="E119" s="79" t="s">
         <v>98</v>
       </c>
@@ -14646,9 +14646,9 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="120" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B120" s="178"/>
-      <c r="D120" s="170"/>
+    <row r="120" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B120" s="164"/>
+      <c r="D120" s="160"/>
       <c r="E120" s="79" t="s">
         <v>98</v>
       </c>
@@ -14747,9 +14747,9 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="121" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B121" s="178"/>
-      <c r="D121" s="170"/>
+    <row r="121" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B121" s="164"/>
+      <c r="D121" s="160"/>
       <c r="E121" s="79" t="s">
         <v>98</v>
       </c>
@@ -14848,9 +14848,9 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="122" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B122" s="178"/>
-      <c r="D122" s="170"/>
+    <row r="122" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B122" s="164"/>
+      <c r="D122" s="160"/>
       <c r="E122" s="79" t="s">
         <v>100</v>
       </c>
@@ -14949,9 +14949,9 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="123" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B123" s="178"/>
-      <c r="D123" s="170"/>
+    <row r="123" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B123" s="164"/>
+      <c r="D123" s="160"/>
       <c r="E123" s="79" t="s">
         <v>100</v>
       </c>
@@ -15050,9 +15050,9 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="124" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B124" s="178"/>
-      <c r="D124" s="170"/>
+    <row r="124" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B124" s="164"/>
+      <c r="D124" s="160"/>
       <c r="E124" s="79" t="s">
         <v>100</v>
       </c>
@@ -15151,9 +15151,9 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="125" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B125" s="178"/>
-      <c r="D125" s="170"/>
+    <row r="125" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B125" s="164"/>
+      <c r="D125" s="160"/>
       <c r="E125" s="79" t="s">
         <v>102</v>
       </c>
@@ -15252,9 +15252,9 @@
         <v>0.41666666666666669</v>
       </c>
     </row>
-    <row r="126" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B126" s="178"/>
-      <c r="D126" s="170"/>
+    <row r="126" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B126" s="164"/>
+      <c r="D126" s="160"/>
       <c r="E126" s="79" t="s">
         <v>102</v>
       </c>
@@ -15353,9 +15353,9 @@
         <v>0.41666666666666669</v>
       </c>
     </row>
-    <row r="127" spans="2:36" x14ac:dyDescent="0.25">
-      <c r="B127" s="178"/>
-      <c r="D127" s="170"/>
+    <row r="127" spans="2:36" x14ac:dyDescent="0.35">
+      <c r="B127" s="164"/>
+      <c r="D127" s="160"/>
       <c r="E127" s="79" t="s">
         <v>102</v>
       </c>
@@ -15454,27 +15454,27 @@
         <v>0.41666666666666669</v>
       </c>
     </row>
-    <row r="128" spans="2:36" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:36" x14ac:dyDescent="0.35">
       <c r="B128" s="87"/>
     </row>
-    <row r="129" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B129" s="171" t="s">
+    <row r="129" spans="2:28" x14ac:dyDescent="0.35">
+      <c r="B129" s="162" t="s">
         <v>111</v>
       </c>
-      <c r="C129" s="145"/>
-      <c r="D129" s="145"/>
-      <c r="E129" s="145"/>
-      <c r="F129" s="145"/>
-      <c r="G129" s="145"/>
-      <c r="H129" s="145"/>
-      <c r="I129" s="145"/>
-      <c r="J129" s="145"/>
-      <c r="K129" s="145"/>
-      <c r="L129" s="145"/>
-      <c r="M129" s="145"/>
-      <c r="N129" s="145"/>
-      <c r="O129" s="145"/>
-      <c r="P129" s="145"/>
+      <c r="C129" s="161"/>
+      <c r="D129" s="161"/>
+      <c r="E129" s="161"/>
+      <c r="F129" s="161"/>
+      <c r="G129" s="161"/>
+      <c r="H129" s="161"/>
+      <c r="I129" s="161"/>
+      <c r="J129" s="161"/>
+      <c r="K129" s="161"/>
+      <c r="L129" s="161"/>
+      <c r="M129" s="161"/>
+      <c r="N129" s="161"/>
+      <c r="O129" s="161"/>
+      <c r="P129" s="161"/>
       <c r="Q129" s="50"/>
       <c r="R129" s="50"/>
       <c r="S129" s="50"/>
@@ -15483,7 +15483,7 @@
       <c r="V129" s="50"/>
       <c r="W129" s="50"/>
     </row>
-    <row r="130" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:28" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B130" s="40"/>
       <c r="C130" s="40"/>
       <c r="D130" s="40"/>
@@ -15507,23 +15507,23 @@
       <c r="V130" s="40"/>
       <c r="W130" s="40"/>
     </row>
-    <row r="131" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B131" s="40"/>
-      <c r="C131" s="172" t="s">
+      <c r="C131" s="152" t="s">
         <v>112</v>
       </c>
-      <c r="D131" s="173"/>
-      <c r="E131" s="173"/>
-      <c r="F131" s="173"/>
-      <c r="G131" s="173"/>
-      <c r="H131" s="173"/>
-      <c r="I131" s="174" t="s">
+      <c r="D131" s="153"/>
+      <c r="E131" s="153"/>
+      <c r="F131" s="153"/>
+      <c r="G131" s="153"/>
+      <c r="H131" s="153"/>
+      <c r="I131" s="155" t="s">
         <v>113</v>
       </c>
-      <c r="J131" s="175"/>
-      <c r="K131" s="175"/>
-      <c r="L131" s="175"/>
-      <c r="M131" s="176"/>
+      <c r="J131" s="156"/>
+      <c r="K131" s="156"/>
+      <c r="L131" s="156"/>
+      <c r="M131" s="157"/>
       <c r="N131" s="89" t="s">
         <v>114</v>
       </c>
@@ -15539,16 +15539,16 @@
       <c r="V131" s="91"/>
       <c r="W131" s="92"/>
     </row>
-    <row r="132" spans="2:28" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:28" ht="14.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B132" s="40"/>
-      <c r="C132" s="162" t="s">
+      <c r="C132" s="142" t="s">
         <v>116</v>
       </c>
-      <c r="D132" s="163"/>
-      <c r="E132" s="163"/>
-      <c r="F132" s="163"/>
-      <c r="G132" s="163"/>
-      <c r="H132" s="164"/>
+      <c r="D132" s="143"/>
+      <c r="E132" s="143"/>
+      <c r="F132" s="143"/>
+      <c r="G132" s="143"/>
+      <c r="H132" s="144"/>
       <c r="I132" t="s">
         <v>93</v>
       </c>
@@ -15557,16 +15557,16 @@
       <c r="O132" s="98"/>
       <c r="W132" s="99"/>
     </row>
-    <row r="133" spans="2:28" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:28" ht="14.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B133" s="40"/>
-      <c r="C133" s="162" t="s">
+      <c r="C133" s="142" t="s">
         <v>117</v>
       </c>
-      <c r="D133" s="163"/>
-      <c r="E133" s="163"/>
-      <c r="F133" s="163"/>
-      <c r="G133" s="163"/>
-      <c r="H133" s="164"/>
+      <c r="D133" s="143"/>
+      <c r="E133" s="143"/>
+      <c r="F133" s="143"/>
+      <c r="G133" s="143"/>
+      <c r="H133" s="144"/>
       <c r="I133" s="100" t="s">
         <v>93</v>
       </c>
@@ -15587,23 +15587,23 @@
       <c r="V133" s="101"/>
       <c r="W133" s="104"/>
     </row>
-    <row r="134" spans="2:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:28" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B134" s="40"/>
-      <c r="C134" s="162" t="s">
+      <c r="C134" s="142" t="s">
         <v>106</v>
       </c>
-      <c r="D134" s="163"/>
-      <c r="E134" s="163"/>
-      <c r="F134" s="163"/>
-      <c r="G134" s="163"/>
-      <c r="H134" s="164"/>
-      <c r="I134" s="165" t="s">
+      <c r="D134" s="143"/>
+      <c r="E134" s="143"/>
+      <c r="F134" s="143"/>
+      <c r="G134" s="143"/>
+      <c r="H134" s="144"/>
+      <c r="I134" s="148" t="s">
         <v>119</v>
       </c>
-      <c r="J134" s="166"/>
-      <c r="K134" s="166"/>
-      <c r="L134" s="166"/>
-      <c r="M134" s="167"/>
+      <c r="J134" s="149"/>
+      <c r="K134" s="149"/>
+      <c r="L134" s="149"/>
+      <c r="M134" s="150"/>
       <c r="N134" s="105"/>
       <c r="O134" s="105"/>
       <c r="P134" s="106"/>
@@ -15615,23 +15615,23 @@
       <c r="V134" s="106"/>
       <c r="W134" s="107"/>
     </row>
-    <row r="135" spans="2:28" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:28" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B135" s="40"/>
-      <c r="C135" s="162" t="s">
+      <c r="C135" s="142" t="s">
         <v>120</v>
       </c>
-      <c r="D135" s="163"/>
-      <c r="E135" s="163"/>
-      <c r="F135" s="163"/>
-      <c r="G135" s="163"/>
-      <c r="H135" s="164"/>
-      <c r="I135" s="165" t="s">
+      <c r="D135" s="143"/>
+      <c r="E135" s="143"/>
+      <c r="F135" s="143"/>
+      <c r="G135" s="143"/>
+      <c r="H135" s="144"/>
+      <c r="I135" s="148" t="s">
         <v>121</v>
       </c>
-      <c r="J135" s="166"/>
-      <c r="K135" s="166"/>
-      <c r="L135" s="166"/>
-      <c r="M135" s="167"/>
+      <c r="J135" s="149"/>
+      <c r="K135" s="149"/>
+      <c r="L135" s="149"/>
+      <c r="M135" s="150"/>
       <c r="N135" s="105"/>
       <c r="O135" s="105"/>
       <c r="P135" s="106"/>
@@ -15643,16 +15643,16 @@
       <c r="V135" s="106"/>
       <c r="W135" s="107"/>
     </row>
-    <row r="136" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B136" s="40"/>
-      <c r="C136" s="162" t="s">
+      <c r="C136" s="142" t="s">
         <v>122</v>
       </c>
-      <c r="D136" s="163"/>
-      <c r="E136" s="163"/>
-      <c r="F136" s="163"/>
-      <c r="G136" s="163"/>
-      <c r="H136" s="164"/>
+      <c r="D136" s="143"/>
+      <c r="E136" s="143"/>
+      <c r="F136" s="143"/>
+      <c r="G136" s="143"/>
+      <c r="H136" s="144"/>
       <c r="I136" s="108" t="s">
         <v>93</v>
       </c>
@@ -15671,16 +15671,16 @@
       <c r="V136" s="109"/>
       <c r="W136" s="111"/>
     </row>
-    <row r="137" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:28" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B137" s="40"/>
-      <c r="C137" s="179" t="s">
+      <c r="C137" s="145" t="s">
         <v>123</v>
       </c>
-      <c r="D137" s="180"/>
-      <c r="E137" s="180"/>
-      <c r="F137" s="180"/>
-      <c r="G137" s="180"/>
-      <c r="H137" s="181"/>
+      <c r="D137" s="146"/>
+      <c r="E137" s="146"/>
+      <c r="F137" s="146"/>
+      <c r="G137" s="146"/>
+      <c r="H137" s="147"/>
       <c r="I137" s="112" t="s">
         <v>93</v>
       </c>
@@ -15699,14 +15699,14 @@
       <c r="V137" s="113"/>
       <c r="W137" s="115"/>
     </row>
-    <row r="138" spans="2:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:28" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B138" s="40"/>
-      <c r="C138" s="182"/>
-      <c r="D138" s="182"/>
-      <c r="E138" s="182"/>
-      <c r="F138" s="182"/>
-      <c r="G138" s="182"/>
-      <c r="H138" s="182"/>
+      <c r="C138" s="151"/>
+      <c r="D138" s="151"/>
+      <c r="E138" s="151"/>
+      <c r="F138" s="151"/>
+      <c r="G138" s="151"/>
+      <c r="H138" s="151"/>
       <c r="I138" s="116"/>
       <c r="J138" s="116"/>
       <c r="K138" s="116"/>
@@ -15723,23 +15723,23 @@
       <c r="V138" s="117"/>
       <c r="W138" s="117"/>
     </row>
-    <row r="139" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B139" s="40"/>
-      <c r="C139" s="172" t="s">
+      <c r="C139" s="152" t="s">
         <v>124</v>
       </c>
-      <c r="D139" s="173"/>
-      <c r="E139" s="173"/>
-      <c r="F139" s="173"/>
-      <c r="G139" s="173"/>
-      <c r="H139" s="183"/>
-      <c r="I139" s="174" t="s">
+      <c r="D139" s="153"/>
+      <c r="E139" s="153"/>
+      <c r="F139" s="153"/>
+      <c r="G139" s="153"/>
+      <c r="H139" s="154"/>
+      <c r="I139" s="155" t="s">
         <v>113</v>
       </c>
-      <c r="J139" s="175"/>
-      <c r="K139" s="175"/>
-      <c r="L139" s="175"/>
-      <c r="M139" s="176"/>
+      <c r="J139" s="156"/>
+      <c r="K139" s="156"/>
+      <c r="L139" s="156"/>
+      <c r="M139" s="157"/>
       <c r="N139" s="89" t="s">
         <v>114</v>
       </c>
@@ -15755,16 +15755,16 @@
       <c r="V139" s="119"/>
       <c r="W139" s="120"/>
     </row>
-    <row r="140" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B140" s="40"/>
-      <c r="C140" s="162" t="s">
+      <c r="C140" s="142" t="s">
         <v>117</v>
       </c>
-      <c r="D140" s="163"/>
-      <c r="E140" s="163"/>
-      <c r="F140" s="163"/>
-      <c r="G140" s="163"/>
-      <c r="H140" s="164"/>
+      <c r="D140" s="143"/>
+      <c r="E140" s="143"/>
+      <c r="F140" s="143"/>
+      <c r="G140" s="143"/>
+      <c r="H140" s="144"/>
       <c r="I140" s="100" t="s">
         <v>93</v>
       </c>
@@ -15785,7 +15785,7 @@
       <c r="V140" s="101"/>
       <c r="W140" s="104"/>
     </row>
-    <row r="141" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B141" s="40"/>
       <c r="C141" s="93" t="s">
         <v>106</v>
@@ -15813,7 +15813,7 @@
       <c r="V141" s="123"/>
       <c r="W141" s="126"/>
     </row>
-    <row r="142" spans="2:28" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:28" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C142" s="93" t="s">
         <v>126</v>
       </c>
@@ -15846,16 +15846,16 @@
       <c r="AA142" s="94"/>
       <c r="AB142" s="95"/>
     </row>
-    <row r="143" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B143" s="40"/>
-      <c r="C143" s="162" t="s">
+      <c r="C143" s="142" t="s">
         <v>120</v>
       </c>
-      <c r="D143" s="163"/>
-      <c r="E143" s="163"/>
-      <c r="F143" s="163"/>
-      <c r="G143" s="163"/>
-      <c r="H143" s="164"/>
+      <c r="D143" s="143"/>
+      <c r="E143" s="143"/>
+      <c r="F143" s="143"/>
+      <c r="G143" s="143"/>
+      <c r="H143" s="144"/>
       <c r="I143" s="122" t="s">
         <v>125</v>
       </c>
@@ -15874,16 +15874,16 @@
       <c r="V143" s="131"/>
       <c r="W143" s="134"/>
     </row>
-    <row r="144" spans="2:28" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B144" s="40"/>
-      <c r="C144" s="162" t="s">
+      <c r="C144" s="142" t="s">
         <v>122</v>
       </c>
-      <c r="D144" s="163"/>
-      <c r="E144" s="163"/>
-      <c r="F144" s="163"/>
-      <c r="G144" s="163"/>
-      <c r="H144" s="164"/>
+      <c r="D144" s="143"/>
+      <c r="E144" s="143"/>
+      <c r="F144" s="143"/>
+      <c r="G144" s="143"/>
+      <c r="H144" s="144"/>
       <c r="I144" s="122" t="s">
         <v>125</v>
       </c>
@@ -15902,16 +15902,16 @@
       <c r="V144" s="109"/>
       <c r="W144" s="111"/>
     </row>
-    <row r="145" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B145" s="40"/>
-      <c r="C145" s="179" t="s">
+      <c r="C145" s="145" t="s">
         <v>128</v>
       </c>
-      <c r="D145" s="180"/>
-      <c r="E145" s="180"/>
-      <c r="F145" s="180"/>
-      <c r="G145" s="180"/>
-      <c r="H145" s="181"/>
+      <c r="D145" s="146"/>
+      <c r="E145" s="146"/>
+      <c r="F145" s="146"/>
+      <c r="G145" s="146"/>
+      <c r="H145" s="147"/>
       <c r="I145" s="112" t="s">
         <v>93</v>
       </c>
@@ -15930,250 +15930,249 @@
       <c r="V145" s="113"/>
       <c r="W145" s="115"/>
     </row>
-    <row r="146" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B146" s="87"/>
     </row>
-    <row r="147" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B147" s="87"/>
     </row>
-    <row r="148" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B148" s="87"/>
     </row>
-    <row r="149" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B149" s="87"/>
     </row>
-    <row r="150" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B150" s="87"/>
     </row>
-    <row r="151" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B151" s="87"/>
     </row>
-    <row r="152" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B152" s="87"/>
     </row>
-    <row r="153" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B153" s="87"/>
     </row>
-    <row r="154" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B154" s="87"/>
     </row>
-    <row r="155" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B155" s="87"/>
     </row>
-    <row r="156" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B156" s="87"/>
     </row>
-    <row r="157" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B157" s="87"/>
     </row>
-    <row r="158" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B158" s="87"/>
     </row>
-    <row r="159" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B159" s="87"/>
     </row>
-    <row r="160" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B160" s="87"/>
     </row>
-    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B161" s="87"/>
     </row>
-    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B162" s="87"/>
     </row>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B163" s="87"/>
     </row>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B164" s="87"/>
     </row>
-    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B165" s="87"/>
     </row>
-    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B166" s="87"/>
     </row>
-    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B167" s="87"/>
     </row>
-    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B168" s="87"/>
     </row>
-    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B169" s="87"/>
     </row>
-    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B170" s="87"/>
     </row>
-    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B171" s="87"/>
     </row>
-    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B172" s="87"/>
     </row>
-    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B173" s="87"/>
     </row>
-    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B174" s="87"/>
     </row>
-    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B175" s="87"/>
     </row>
-    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B176" s="87"/>
     </row>
-    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B177" s="87"/>
     </row>
-    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B178" s="87"/>
     </row>
-    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B179" s="87"/>
     </row>
-    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B180" s="87"/>
     </row>
-    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B181" s="87"/>
     </row>
-    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B182" s="87"/>
     </row>
-    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B183" s="87"/>
     </row>
-    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B184" s="87"/>
     </row>
-    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B185" s="87"/>
     </row>
-    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B186" s="87"/>
     </row>
-    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B187" s="87"/>
     </row>
-    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B188" s="87"/>
     </row>
-    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B189" s="87"/>
     </row>
-    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B190" s="87"/>
     </row>
-    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B191" s="87"/>
     </row>
-    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B192" s="87"/>
     </row>
-    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B193" s="87"/>
     </row>
-    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B194" s="87"/>
     </row>
-    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B195" s="87"/>
     </row>
-    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B196" s="87"/>
     </row>
-    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B197" s="87"/>
     </row>
-    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B198" s="87"/>
     </row>
-    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B199" s="87"/>
     </row>
-    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="200" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B200" s="87"/>
     </row>
-    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="201" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B201" s="87"/>
     </row>
-    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="202" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B202" s="87"/>
     </row>
-    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="203" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B203" s="87"/>
     </row>
-    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="204" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B204" s="87"/>
     </row>
-    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="205" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B205" s="87"/>
     </row>
-    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="206" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B206" s="87"/>
     </row>
-    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="207" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B207" s="87"/>
     </row>
-    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="208" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B208" s="87"/>
     </row>
-    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="209" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B209" s="87"/>
     </row>
-    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="210" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B210" s="87"/>
     </row>
-    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="211" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B211" s="87"/>
     </row>
-    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="212" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B212" s="87"/>
     </row>
-    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="213" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B213" s="87"/>
     </row>
-    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="214" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B214" s="87"/>
     </row>
-    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="215" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B215" s="87"/>
     </row>
-    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="216" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B216" s="87"/>
     </row>
-    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="217" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B217" s="87"/>
     </row>
-    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="218" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B218" s="87"/>
     </row>
-    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="219" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B219" s="87"/>
     </row>
-    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="220" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B220" s="87"/>
     </row>
-    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="221" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B221" s="87"/>
     </row>
-    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="222" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B222" s="87"/>
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="C140:H140"/>
-    <mergeCell ref="C143:H143"/>
-    <mergeCell ref="C144:H144"/>
-    <mergeCell ref="C145:H145"/>
-    <mergeCell ref="C135:H135"/>
-    <mergeCell ref="I135:M135"/>
-    <mergeCell ref="C136:H136"/>
-    <mergeCell ref="C137:H137"/>
-    <mergeCell ref="C138:H138"/>
-    <mergeCell ref="C139:H139"/>
-    <mergeCell ref="I139:M139"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="C7:Q7"/>
+    <mergeCell ref="B9:B36"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:L9"/>
+    <mergeCell ref="D11:L11"/>
+    <mergeCell ref="D12:L12"/>
+    <mergeCell ref="D13:L13"/>
+    <mergeCell ref="C15:P16"/>
     <mergeCell ref="C134:H134"/>
     <mergeCell ref="I134:M134"/>
     <mergeCell ref="D17:D27"/>
@@ -16190,16 +16189,17 @@
     <mergeCell ref="D79:D93"/>
     <mergeCell ref="D96:D110"/>
     <mergeCell ref="D113:D127"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="C7:Q7"/>
-    <mergeCell ref="B9:B36"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:L9"/>
-    <mergeCell ref="D11:L11"/>
-    <mergeCell ref="D12:L12"/>
-    <mergeCell ref="D13:L13"/>
-    <mergeCell ref="C15:P16"/>
+    <mergeCell ref="I135:M135"/>
+    <mergeCell ref="C136:H136"/>
+    <mergeCell ref="C137:H137"/>
+    <mergeCell ref="C138:H138"/>
+    <mergeCell ref="C139:H139"/>
+    <mergeCell ref="I139:M139"/>
+    <mergeCell ref="C140:H140"/>
+    <mergeCell ref="C143:H143"/>
+    <mergeCell ref="C144:H144"/>
+    <mergeCell ref="C145:H145"/>
+    <mergeCell ref="C135:H135"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="M1" r:id="rId1" display="https://atb.nrel.gov/electricity/2022/utility-scale_battery_storage" xr:uid="{7816EC9A-0454-4087-A6E1-F971C99AA20E}"/>
@@ -16216,13 +16216,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC34B27C-0BFA-4D35-874E-EA84BA74EBE0}">
   <dimension ref="A1:N28"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="32.5703125" customWidth="1"/>
-    <col min="2" max="14" width="11.28515625" customWidth="1"/>
+    <col min="1" max="1" width="32.54296875" customWidth="1"/>
+    <col min="2" max="14" width="11.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="32" t="s">
         <v>19</v>
       </c>
@@ -16240,7 +16240,7 @@
       <c r="M1" s="33"/>
       <c r="N1" s="33"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="15"/>
       <c r="B2" s="184" t="s">
         <v>20</v>
@@ -16264,7 +16264,7 @@
       <c r="M2" s="185"/>
       <c r="N2" s="186"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="18" t="s">
         <v>41</v>
       </c>
@@ -16306,7 +16306,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="16" t="s">
         <v>24</v>
       </c>
@@ -16351,7 +16351,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="16" t="s">
         <v>25</v>
       </c>
@@ -16396,7 +16396,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="16" t="s">
         <v>26</v>
       </c>
@@ -16441,7 +16441,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="16" t="s">
         <v>27</v>
       </c>
@@ -16486,7 +16486,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="16" t="s">
         <v>42</v>
       </c>
@@ -16531,7 +16531,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="16" t="s">
         <v>28</v>
       </c>
@@ -16576,7 +16576,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
         <v>29</v>
       </c>
@@ -16621,7 +16621,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="22" t="s">
         <v>30</v>
       </c>
@@ -16666,7 +16666,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="17" t="s">
         <v>31</v>
       </c>
@@ -16708,7 +16708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="16" t="s">
         <v>32</v>
       </c>
@@ -16750,7 +16750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="16" t="s">
         <v>33</v>
       </c>
@@ -16792,7 +16792,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="16" t="s">
         <v>34</v>
       </c>
@@ -16834,7 +16834,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
         <v>35</v>
       </c>
@@ -16876,7 +16876,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="16" t="s">
         <v>36</v>
       </c>
@@ -16918,7 +16918,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" s="27" t="s">
         <v>37</v>
       </c>
@@ -16960,12 +16960,12 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" s="34" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>49</v>
       </c>
@@ -16978,7 +16978,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>50</v>
       </c>
@@ -16991,7 +16991,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>18</v>
       </c>
@@ -17004,7 +17004,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>18</v>
       </c>
@@ -17017,7 +17017,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -17030,7 +17030,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>60</v>
       </c>
@@ -17050,12 +17050,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD9A83FF-6D12-451D-B709-5F68973469C6}">
   <dimension ref="A1:AE12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="47" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>144</v>
       </c>
@@ -17150,7 +17150,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>149</v>
       </c>
@@ -17245,13 +17245,13 @@
         <v>137190</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="C3">
         <f>C9*$B$12*1000</f>
         <v>306878.94936720002</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="C3:AE3" si="0">D9*$B$12*1000</f>
+        <f t="shared" ref="D3:AE3" si="0">D9*$B$12*1000</f>
         <v>303731.66899460001</v>
       </c>
       <c r="E3">
@@ -17363,7 +17363,7 @@
         <v>123431.08661402132</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>144</v>
       </c>
@@ -17458,7 +17458,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>151</v>
       </c>
@@ -17553,7 +17553,7 @@
         <v>212064</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="C7">
         <f t="shared" ref="C7:AE7" si="1">C10*$B$12*1000</f>
         <v>284959.40253119997</v>
@@ -17671,7 +17671,7 @@
         <v>212193.12422562522</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>143</v>
       </c>
@@ -17766,7 +17766,7 @@
         <v>157.23705301149212</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>143</v>
       </c>
@@ -17861,7 +17861,7 @@
         <v>270.30971238933148</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>150</v>
       </c>
@@ -17881,14 +17881,14 @@
     <tabColor rgb="FF003399"/>
   </sheetPr>
   <dimension ref="A1:G31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="2" max="2" width="21.42578125" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -17896,7 +17896,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -17907,7 +17907,7 @@
       <c r="E2" s="5"/>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2022</v>
       </c>
@@ -17917,7 +17917,7 @@
       </c>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2023</v>
       </c>
@@ -17926,15 +17926,16 @@
         <v>303546.34355618269</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2024</v>
       </c>
       <c r="B5" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <f>'NREL ATB 2024'!I20*1000*cpi_2022_to_2012</f>
+        <v>279096.37947464635</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2025</v>
       </c>
@@ -17942,7 +17943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -17950,7 +17951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2027</v>
       </c>
@@ -17958,7 +17959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2028</v>
       </c>
@@ -17966,7 +17967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2029</v>
       </c>
@@ -17974,7 +17975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2030</v>
       </c>
@@ -17982,7 +17983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2031</v>
       </c>
@@ -17990,7 +17991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2032</v>
       </c>
@@ -17998,7 +17999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2033</v>
       </c>
@@ -18006,7 +18007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>2034</v>
       </c>
@@ -18014,7 +18015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>2035</v>
       </c>
@@ -18022,7 +18023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2036</v>
       </c>
@@ -18030,7 +18031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2037</v>
       </c>
@@ -18038,7 +18039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2038</v>
       </c>
@@ -18046,7 +18047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2039</v>
       </c>
@@ -18054,7 +18055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2040</v>
       </c>
@@ -18062,7 +18063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2041</v>
       </c>
@@ -18070,7 +18071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2042</v>
       </c>
@@ -18078,7 +18079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2043</v>
       </c>
@@ -18086,7 +18087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2044</v>
       </c>
@@ -18094,7 +18095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2045</v>
       </c>
@@ -18102,7 +18103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2046</v>
       </c>
@@ -18110,7 +18111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2047</v>
       </c>
@@ -18118,7 +18119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2048</v>
       </c>
@@ -18126,7 +18127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2049</v>
       </c>
@@ -18134,7 +18135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2050</v>
       </c>
@@ -18153,14 +18154,14 @@
     <tabColor rgb="FF003399"/>
   </sheetPr>
   <dimension ref="A1:G31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="2" max="2" width="21.42578125" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -18168,7 +18169,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2021</v>
       </c>
@@ -18178,7 +18179,7 @@
       </c>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2022</v>
       </c>
@@ -18187,7 +18188,7 @@
         <v>284785.53121122846</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2023</v>
       </c>
@@ -18196,7 +18197,7 @@
         <v>281864.83588615071</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2024</v>
       </c>
@@ -18205,7 +18206,7 @@
         <v>272119.91517411894</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2025</v>
       </c>
@@ -18214,7 +18215,7 @@
         <v>244267.93200601047</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -18223,7 +18224,7 @@
         <v>245045.09148289612</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2027</v>
       </c>
@@ -18232,7 +18233,7 @@
         <v>245896.5501406297</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2028</v>
       </c>
@@ -18241,7 +18242,7 @@
         <v>246831.28958028281</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2029</v>
       </c>
@@ -18250,7 +18251,7 @@
         <v>247859.79983015926</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2030</v>
       </c>
@@ -18259,7 +18260,7 @@
         <v>248994.40989292334</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2031</v>
       </c>
@@ -18268,7 +18269,7 @@
         <v>247303.59777741029</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2032</v>
       </c>
@@ -18277,7 +18278,7 @@
         <v>245600.17607833183</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2033</v>
       </c>
@@ -18286,7 +18287,7 @@
         <v>243883.65354072856</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>2034</v>
       </c>
@@ -18295,7 +18296,7 @@
         <v>242153.5130555816</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>2035</v>
       </c>
@@ -18304,7 +18305,7 @@
         <v>240409.20993631281</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2036</v>
       </c>
@@ -18313,7 +18314,7 @@
         <v>238650.17005554074</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2037</v>
       </c>
@@ -18322,7 +18323,7 @@
         <v>236875.78782870833</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2038</v>
       </c>
@@ -18331,7 +18332,7 @@
         <v>235085.42402968768</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2039</v>
       </c>
@@ -18340,7 +18341,7 @@
         <v>233278.40342179779</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2040</v>
       </c>
@@ -18349,7 +18350,7 @@
         <v>231454.01218578266</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2041</v>
       </c>
@@ -18358,7 +18359,7 @@
         <v>229611.49512414529</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2042</v>
       </c>
@@ -18367,7 +18368,7 @@
         <v>227750.05261882479</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2043</v>
       </c>
@@ -18376,7 +18377,7 @@
         <v>225868.83731644039</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2044</v>
       </c>
@@ -18385,7 +18386,7 @@
         <v>223966.95051221756</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2045</v>
       </c>
@@ -18394,7 +18395,7 @@
         <v>222043.43820014191</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2046</v>
       </c>
@@ -18403,7 +18404,7 @@
         <v>220097.2867528405</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2047</v>
       </c>
@@ -18412,7 +18413,7 @@
         <v>218127.41819005259</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2048</v>
       </c>
@@ -18421,7 +18422,7 @@
         <v>216132.68498924136</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2049</v>
       </c>
@@ -18430,7 +18431,7 @@
         <v>214111.864385811</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2050</v>
       </c>
@@ -18450,12 +18451,12 @@
     <tabColor rgb="FF003399"/>
   </sheetPr>
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>130</v>
       </c>
@@ -18463,7 +18464,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>131</v>
       </c>

</xml_diff>

<commit_message>
Make BBoSCaSoFYC time series to address issue #327
</commit_message>
<xml_diff>
--- a/InputData/elec/BCpUC/Battery Cost per Unit Cap.xlsx
+++ b/InputData/elec/BCpUC/Battery Cost per Unit Cap.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BCpUC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4D004E-9358-4857-BE9A-195C5BF97CD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{284B9C25-D938-4BAA-984B-FCB62253D7AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="839" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="151">
   <si>
     <t>Year</t>
   </si>
@@ -452,9 +452,6 @@
   </si>
   <si>
     <t>Unit: Dmnl</t>
-  </si>
-  <si>
-    <t>Percent of First Year Total Costs</t>
   </si>
   <si>
     <t>Assumed duration:</t>
@@ -1971,69 +1968,15 @@
     <xf numFmtId="5" fontId="10" fillId="14" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="169" fontId="10" fillId="14" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="59" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
@@ -2080,6 +2023,60 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="58" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="59" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4627,7 +4624,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -4715,7 +4712,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
@@ -4760,12 +4757,12 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
@@ -4775,12 +4772,12 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
@@ -4790,7 +4787,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
@@ -4805,7 +4802,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
@@ -4855,7 +4852,7 @@
         <v>0.84730412960844359</v>
       </c>
       <c r="B51" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C51">
         <f>cpi_2022_to_2012/A51</f>
@@ -4867,7 +4864,7 @@
         <v>0.78452102304761584</v>
       </c>
       <c r="B52" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
@@ -4877,7 +4874,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B55">
         <v>4</v>
@@ -4908,19 +4905,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:108" s="40" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A1" s="165" t="s">
+      <c r="A1" s="142" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="165"/>
-      <c r="C1" s="165"/>
-      <c r="D1" s="165"/>
-      <c r="E1" s="165"/>
-      <c r="F1" s="165"/>
-      <c r="G1" s="165"/>
-      <c r="H1" s="165"/>
-      <c r="I1" s="165"/>
-      <c r="J1" s="165"/>
-      <c r="K1" s="165"/>
+      <c r="B1" s="142"/>
+      <c r="C1" s="142"/>
+      <c r="D1" s="142"/>
+      <c r="E1" s="142"/>
+      <c r="F1" s="142"/>
+      <c r="G1" s="142"/>
+      <c r="H1" s="142"/>
+      <c r="I1" s="142"/>
+      <c r="J1" s="142"/>
+      <c r="K1" s="142"/>
       <c r="M1" s="3" t="s">
         <v>68</v>
       </c>
@@ -5050,12 +5047,12 @@
     </row>
     <row r="4" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D4" s="44"/>
-      <c r="L4" s="166" t="s">
+      <c r="L4" s="143" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:108" ht="14.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="L5" s="167"/>
+      <c r="L5" s="144"/>
     </row>
     <row r="6" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H6" s="45"/>
@@ -5087,23 +5084,23 @@
       <c r="B7" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="161" t="s">
+      <c r="C7" s="145" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="161"/>
-      <c r="E7" s="161"/>
-      <c r="F7" s="161"/>
-      <c r="G7" s="161"/>
-      <c r="H7" s="161"/>
-      <c r="I7" s="161"/>
-      <c r="J7" s="161"/>
-      <c r="K7" s="161"/>
-      <c r="L7" s="161"/>
-      <c r="M7" s="161"/>
-      <c r="N7" s="161"/>
-      <c r="O7" s="161"/>
-      <c r="P7" s="161"/>
-      <c r="Q7" s="161"/>
+      <c r="D7" s="145"/>
+      <c r="E7" s="145"/>
+      <c r="F7" s="145"/>
+      <c r="G7" s="145"/>
+      <c r="H7" s="145"/>
+      <c r="I7" s="145"/>
+      <c r="J7" s="145"/>
+      <c r="K7" s="145"/>
+      <c r="L7" s="145"/>
+      <c r="M7" s="145"/>
+      <c r="N7" s="145"/>
+      <c r="O7" s="145"/>
+      <c r="P7" s="145"/>
+      <c r="Q7" s="145"/>
       <c r="R7" s="50"/>
       <c r="S7" s="50"/>
       <c r="T7" s="50"/>
@@ -5121,43 +5118,43 @@
     </row>
     <row r="9" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9"/>
-      <c r="B9" s="168" t="s">
+      <c r="B9" s="146" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="169" t="s">
+      <c r="D9" s="147" t="s">
         <v>75</v>
       </c>
-      <c r="E9" s="170"/>
-      <c r="F9" s="171"/>
-      <c r="G9" s="172">
+      <c r="E9" s="148"/>
+      <c r="F9" s="149"/>
+      <c r="G9" s="150">
         <v>2022</v>
       </c>
-      <c r="H9" s="173"/>
-      <c r="I9" s="173"/>
-      <c r="J9" s="173"/>
-      <c r="K9" s="174"/>
-      <c r="L9" s="174"/>
+      <c r="H9" s="151"/>
+      <c r="I9" s="151"/>
+      <c r="J9" s="151"/>
+      <c r="K9" s="152"/>
+      <c r="L9" s="152"/>
     </row>
     <row r="10" spans="1:108" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="168"/>
+      <c r="B10" s="146"/>
       <c r="D10" s="53" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J10" s="52"/>
     </row>
     <row r="11" spans="1:108" s="40" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="168"/>
-      <c r="D11" s="175" t="s">
+      <c r="B11" s="146"/>
+      <c r="D11" s="153" t="s">
         <v>76</v>
       </c>
-      <c r="E11" s="176"/>
-      <c r="F11" s="176"/>
-      <c r="G11" s="176"/>
-      <c r="H11" s="176"/>
-      <c r="I11" s="176"/>
-      <c r="J11" s="176"/>
-      <c r="K11" s="176"/>
-      <c r="L11" s="176"/>
+      <c r="E11" s="154"/>
+      <c r="F11" s="154"/>
+      <c r="G11" s="154"/>
+      <c r="H11" s="154"/>
+      <c r="I11" s="154"/>
+      <c r="J11" s="154"/>
+      <c r="K11" s="154"/>
+      <c r="L11" s="154"/>
       <c r="W11" s="54"/>
       <c r="X11" s="55"/>
       <c r="Y11" s="55"/>
@@ -5165,18 +5162,18 @@
       <c r="AA11" s="55"/>
     </row>
     <row r="12" spans="1:108" s="40" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="168"/>
-      <c r="D12" s="177" t="s">
+      <c r="B12" s="146"/>
+      <c r="D12" s="155" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="178"/>
-      <c r="F12" s="178"/>
-      <c r="G12" s="178"/>
-      <c r="H12" s="178"/>
-      <c r="I12" s="178"/>
-      <c r="J12" s="178"/>
-      <c r="K12" s="178"/>
-      <c r="L12" s="179"/>
+      <c r="E12" s="156"/>
+      <c r="F12" s="156"/>
+      <c r="G12" s="156"/>
+      <c r="H12" s="156"/>
+      <c r="I12" s="156"/>
+      <c r="J12" s="156"/>
+      <c r="K12" s="156"/>
+      <c r="L12" s="157"/>
       <c r="M12" s="56"/>
       <c r="W12" s="54"/>
       <c r="X12" s="55"/>
@@ -5185,16 +5182,16 @@
       <c r="AA12" s="55"/>
     </row>
     <row r="13" spans="1:108" s="40" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="168"/>
-      <c r="D13" s="180"/>
-      <c r="E13" s="181"/>
-      <c r="F13" s="181"/>
-      <c r="G13" s="181"/>
-      <c r="H13" s="181"/>
-      <c r="I13" s="181"/>
-      <c r="J13" s="181"/>
-      <c r="K13" s="181"/>
-      <c r="L13" s="182"/>
+      <c r="B13" s="146"/>
+      <c r="D13" s="158"/>
+      <c r="E13" s="159"/>
+      <c r="F13" s="159"/>
+      <c r="G13" s="159"/>
+      <c r="H13" s="159"/>
+      <c r="I13" s="159"/>
+      <c r="J13" s="159"/>
+      <c r="K13" s="159"/>
+      <c r="L13" s="160"/>
       <c r="W13" s="54"/>
       <c r="X13" s="55"/>
       <c r="Y13" s="55"/>
@@ -5202,49 +5199,49 @@
       <c r="AA13" s="55"/>
     </row>
     <row r="14" spans="1:108" ht="37.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="168"/>
+      <c r="B14" s="146"/>
     </row>
     <row r="15" spans="1:108" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="168"/>
-      <c r="C15" s="183" t="s">
-        <v>147</v>
-      </c>
-      <c r="D15" s="183"/>
-      <c r="E15" s="183"/>
-      <c r="F15" s="183"/>
-      <c r="G15" s="183"/>
-      <c r="H15" s="183"/>
-      <c r="I15" s="183"/>
-      <c r="J15" s="183"/>
-      <c r="K15" s="183"/>
-      <c r="L15" s="183"/>
-      <c r="M15" s="183"/>
-      <c r="N15" s="183"/>
-      <c r="O15" s="183"/>
-      <c r="P15" s="183"/>
+      <c r="B15" s="146"/>
+      <c r="C15" s="161" t="s">
+        <v>146</v>
+      </c>
+      <c r="D15" s="161"/>
+      <c r="E15" s="161"/>
+      <c r="F15" s="161"/>
+      <c r="G15" s="161"/>
+      <c r="H15" s="161"/>
+      <c r="I15" s="161"/>
+      <c r="J15" s="161"/>
+      <c r="K15" s="161"/>
+      <c r="L15" s="161"/>
+      <c r="M15" s="161"/>
+      <c r="N15" s="161"/>
+      <c r="O15" s="161"/>
+      <c r="P15" s="161"/>
       <c r="Q15" s="57"/>
     </row>
     <row r="16" spans="1:108" x14ac:dyDescent="0.35">
-      <c r="B16" s="168"/>
-      <c r="C16" s="183"/>
-      <c r="D16" s="183"/>
-      <c r="E16" s="183"/>
-      <c r="F16" s="183"/>
-      <c r="G16" s="183"/>
-      <c r="H16" s="183"/>
-      <c r="I16" s="183"/>
-      <c r="J16" s="183"/>
-      <c r="K16" s="183"/>
-      <c r="L16" s="183"/>
-      <c r="M16" s="183"/>
-      <c r="N16" s="183"/>
-      <c r="O16" s="183"/>
-      <c r="P16" s="183"/>
+      <c r="B16" s="146"/>
+      <c r="C16" s="161"/>
+      <c r="D16" s="161"/>
+      <c r="E16" s="161"/>
+      <c r="F16" s="161"/>
+      <c r="G16" s="161"/>
+      <c r="H16" s="161"/>
+      <c r="I16" s="161"/>
+      <c r="J16" s="161"/>
+      <c r="K16" s="161"/>
+      <c r="L16" s="161"/>
+      <c r="M16" s="161"/>
+      <c r="N16" s="161"/>
+      <c r="O16" s="161"/>
+      <c r="P16" s="161"/>
     </row>
     <row r="17" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="168"/>
+      <c r="B17" s="146"/>
       <c r="C17" s="58"/>
-      <c r="D17" s="158" t="s">
+      <c r="D17" s="168" t="s">
         <v>78</v>
       </c>
       <c r="E17" s="1" t="s">
@@ -5252,11 +5249,11 @@
       </c>
     </row>
     <row r="18" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="168"/>
+      <c r="B18" s="146"/>
       <c r="C18" s="58"/>
-      <c r="D18" s="159"/>
+      <c r="D18" s="169"/>
       <c r="F18" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G18" s="1">
         <v>2022</v>
@@ -5347,9 +5344,9 @@
       </c>
     </row>
     <row r="19" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="168"/>
+      <c r="B19" s="146"/>
       <c r="C19" s="58"/>
-      <c r="D19" s="159"/>
+      <c r="D19" s="169"/>
       <c r="E19" t="s">
         <v>80</v>
       </c>
@@ -5445,9 +5442,9 @@
       </c>
     </row>
     <row r="20" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="168"/>
+      <c r="B20" s="146"/>
       <c r="C20" s="58"/>
-      <c r="D20" s="160"/>
+      <c r="D20" s="170"/>
       <c r="E20" t="s">
         <v>81</v>
       </c>
@@ -5543,9 +5540,9 @@
       </c>
     </row>
     <row r="21" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="168"/>
+      <c r="B21" s="146"/>
       <c r="C21" s="58"/>
-      <c r="D21" s="160"/>
+      <c r="D21" s="170"/>
       <c r="E21" t="s">
         <v>82</v>
       </c>
@@ -5641,9 +5638,9 @@
       </c>
     </row>
     <row r="22" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="168"/>
+      <c r="B22" s="146"/>
       <c r="C22" s="58"/>
-      <c r="D22" s="160"/>
+      <c r="D22" s="170"/>
       <c r="F22" s="60"/>
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
@@ -5676,20 +5673,20 @@
       <c r="AI22" s="5"/>
     </row>
     <row r="23" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="168"/>
+      <c r="B23" s="146"/>
       <c r="C23" s="58"/>
-      <c r="D23" s="160"/>
+      <c r="D23" s="170"/>
       <c r="E23" s="1" t="s">
         <v>83</v>
       </c>
       <c r="F23" s="60"/>
     </row>
     <row r="24" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="168"/>
+      <c r="B24" s="146"/>
       <c r="C24" s="58"/>
-      <c r="D24" s="160"/>
+      <c r="D24" s="170"/>
       <c r="F24" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G24" s="1">
         <v>2022</v>
@@ -5780,9 +5777,9 @@
       </c>
     </row>
     <row r="25" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="168"/>
+      <c r="B25" s="146"/>
       <c r="C25" s="58"/>
-      <c r="D25" s="160"/>
+      <c r="D25" s="170"/>
       <c r="E25" t="s">
         <v>80</v>
       </c>
@@ -5878,9 +5875,9 @@
       </c>
     </row>
     <row r="26" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="168"/>
+      <c r="B26" s="146"/>
       <c r="C26" s="58"/>
-      <c r="D26" s="160"/>
+      <c r="D26" s="170"/>
       <c r="E26" t="s">
         <v>81</v>
       </c>
@@ -5976,9 +5973,9 @@
       </c>
     </row>
     <row r="27" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="168"/>
+      <c r="B27" s="146"/>
       <c r="C27" s="58"/>
-      <c r="D27" s="160"/>
+      <c r="D27" s="170"/>
       <c r="E27" t="s">
         <v>82</v>
       </c>
@@ -6074,7 +6071,7 @@
       </c>
     </row>
     <row r="28" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="168"/>
+      <c r="B28" s="146"/>
       <c r="C28" s="58"/>
       <c r="D28" s="58"/>
       <c r="G28" s="5"/>
@@ -6112,7 +6109,7 @@
       <c r="AM28" s="5"/>
     </row>
     <row r="29" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="168"/>
+      <c r="B29" s="146"/>
       <c r="C29" s="58"/>
       <c r="D29" s="58"/>
       <c r="E29" s="1" t="s">
@@ -6154,7 +6151,7 @@
       <c r="AM29" s="5"/>
     </row>
     <row r="30" spans="2:39" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="168"/>
+      <c r="B30" s="146"/>
       <c r="C30" s="58"/>
       <c r="D30" s="58"/>
       <c r="E30" s="1"/>
@@ -6194,9 +6191,9 @@
       <c r="AM30" s="5"/>
     </row>
     <row r="31" spans="2:39" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B31" s="168"/>
+      <c r="B31" s="146"/>
       <c r="C31" s="58"/>
-      <c r="D31" s="159" t="s">
+      <c r="D31" s="169" t="s">
         <v>85</v>
       </c>
       <c r="E31" s="61" t="s">
@@ -6246,9 +6243,9 @@
       <c r="AM31" s="5"/>
     </row>
     <row r="32" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="168"/>
+      <c r="B32" s="146"/>
       <c r="C32" s="58"/>
-      <c r="D32" s="159"/>
+      <c r="D32" s="169"/>
       <c r="E32" s="66" t="s">
         <v>91</v>
       </c>
@@ -6296,9 +6293,9 @@
       <c r="AM32" s="5"/>
     </row>
     <row r="33" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="168"/>
+      <c r="B33" s="146"/>
       <c r="C33" s="58"/>
-      <c r="D33" s="159"/>
+      <c r="D33" s="169"/>
       <c r="E33" s="69" t="s">
         <v>96</v>
       </c>
@@ -6346,9 +6343,9 @@
       <c r="AM33" s="5"/>
     </row>
     <row r="34" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="168"/>
+      <c r="B34" s="146"/>
       <c r="C34" s="58"/>
-      <c r="D34" s="159"/>
+      <c r="D34" s="169"/>
       <c r="E34" s="72" t="s">
         <v>98</v>
       </c>
@@ -6396,9 +6393,9 @@
       <c r="AM34" s="5"/>
     </row>
     <row r="35" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="168"/>
+      <c r="B35" s="146"/>
       <c r="C35" s="58"/>
-      <c r="D35" s="159"/>
+      <c r="D35" s="169"/>
       <c r="E35" s="69" t="s">
         <v>100</v>
       </c>
@@ -6446,9 +6443,9 @@
       <c r="AM35" s="5"/>
     </row>
     <row r="36" spans="2:74" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B36" s="168"/>
+      <c r="B36" s="146"/>
       <c r="C36" s="58"/>
-      <c r="D36" s="159"/>
+      <c r="D36" s="169"/>
       <c r="E36" s="75" t="s">
         <v>102</v>
       </c>
@@ -6535,23 +6532,23 @@
       <c r="AM37" s="5"/>
     </row>
     <row r="38" spans="2:74" s="40" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C38" s="161" t="s">
+      <c r="C38" s="145" t="s">
         <v>104</v>
       </c>
-      <c r="D38" s="161"/>
-      <c r="E38" s="161"/>
-      <c r="F38" s="161"/>
-      <c r="G38" s="161"/>
-      <c r="H38" s="161"/>
-      <c r="I38" s="161"/>
-      <c r="J38" s="161"/>
-      <c r="K38" s="161"/>
-      <c r="L38" s="161"/>
-      <c r="M38" s="161"/>
-      <c r="N38" s="161"/>
-      <c r="O38" s="161"/>
-      <c r="P38" s="161"/>
-      <c r="Q38" s="161"/>
+      <c r="D38" s="145"/>
+      <c r="E38" s="145"/>
+      <c r="F38" s="145"/>
+      <c r="G38" s="145"/>
+      <c r="H38" s="145"/>
+      <c r="I38" s="145"/>
+      <c r="J38" s="145"/>
+      <c r="K38" s="145"/>
+      <c r="L38" s="145"/>
+      <c r="M38" s="145"/>
+      <c r="N38" s="145"/>
+      <c r="O38" s="145"/>
+      <c r="P38" s="145"/>
+      <c r="Q38" s="145"/>
       <c r="R38" s="50"/>
       <c r="S38" s="50"/>
       <c r="T38" s="50"/>
@@ -6583,7 +6580,7 @@
     <row r="39" spans="2:74" s="40" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="40" spans="2:74" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D40" s="53" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="41" spans="2:74" x14ac:dyDescent="0.35">
@@ -6593,7 +6590,7 @@
     </row>
     <row r="42" spans="2:74" x14ac:dyDescent="0.35">
       <c r="G42" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H42" s="1">
         <v>2022</v>
@@ -6684,10 +6681,10 @@
       </c>
     </row>
     <row r="43" spans="2:74" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B43" s="163" t="s">
+      <c r="B43" s="177" t="s">
         <v>61</v>
       </c>
-      <c r="D43" s="158" t="s">
+      <c r="D43" s="168" t="s">
         <v>106</v>
       </c>
       <c r="E43" s="79" t="s">
@@ -6789,8 +6786,8 @@
       </c>
     </row>
     <row r="44" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B44" s="163"/>
-      <c r="D44" s="159"/>
+      <c r="B44" s="177"/>
+      <c r="D44" s="169"/>
       <c r="E44" s="82" t="s">
         <v>91</v>
       </c>
@@ -6890,8 +6887,8 @@
       </c>
     </row>
     <row r="45" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B45" s="163"/>
-      <c r="D45" s="159"/>
+      <c r="B45" s="177"/>
+      <c r="D45" s="169"/>
       <c r="E45" s="83" t="s">
         <v>91</v>
       </c>
@@ -6991,8 +6988,8 @@
       </c>
     </row>
     <row r="46" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B46" s="163"/>
-      <c r="D46" s="160"/>
+      <c r="B46" s="177"/>
+      <c r="D46" s="170"/>
       <c r="E46" s="79" t="s">
         <v>96</v>
       </c>
@@ -7125,8 +7122,8 @@
       <c r="BV46" s="5"/>
     </row>
     <row r="47" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B47" s="163"/>
-      <c r="D47" s="160"/>
+      <c r="B47" s="177"/>
+      <c r="D47" s="170"/>
       <c r="E47" s="79" t="s">
         <v>96</v>
       </c>
@@ -7259,8 +7256,8 @@
       <c r="BV47" s="5"/>
     </row>
     <row r="48" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B48" s="163"/>
-      <c r="D48" s="160"/>
+      <c r="B48" s="177"/>
+      <c r="D48" s="170"/>
       <c r="E48" s="79" t="s">
         <v>96</v>
       </c>
@@ -7393,8 +7390,8 @@
       <c r="BV48" s="5"/>
     </row>
     <row r="49" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B49" s="163"/>
-      <c r="D49" s="160"/>
+      <c r="B49" s="177"/>
+      <c r="D49" s="170"/>
       <c r="E49" s="79" t="s">
         <v>98</v>
       </c>
@@ -7527,8 +7524,8 @@
       <c r="BV49" s="5"/>
     </row>
     <row r="50" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B50" s="163"/>
-      <c r="D50" s="160"/>
+      <c r="B50" s="177"/>
+      <c r="D50" s="170"/>
       <c r="E50" s="79" t="s">
         <v>98</v>
       </c>
@@ -7661,8 +7658,8 @@
       <c r="BV50" s="5"/>
     </row>
     <row r="51" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B51" s="163"/>
-      <c r="D51" s="160"/>
+      <c r="B51" s="177"/>
+      <c r="D51" s="170"/>
       <c r="E51" s="79" t="s">
         <v>98</v>
       </c>
@@ -7795,8 +7792,8 @@
       <c r="BV51" s="5"/>
     </row>
     <row r="52" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B52" s="163"/>
-      <c r="D52" s="160"/>
+      <c r="B52" s="177"/>
+      <c r="D52" s="170"/>
       <c r="E52" s="79" t="s">
         <v>100</v>
       </c>
@@ -7929,8 +7926,8 @@
       <c r="BV52" s="5"/>
     </row>
     <row r="53" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B53" s="163"/>
-      <c r="D53" s="160"/>
+      <c r="B53" s="177"/>
+      <c r="D53" s="170"/>
       <c r="E53" s="79" t="s">
         <v>100</v>
       </c>
@@ -8063,8 +8060,8 @@
       <c r="BV53" s="5"/>
     </row>
     <row r="54" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B54" s="163"/>
-      <c r="D54" s="160"/>
+      <c r="B54" s="177"/>
+      <c r="D54" s="170"/>
       <c r="E54" s="79" t="s">
         <v>100</v>
       </c>
@@ -8197,8 +8194,8 @@
       <c r="BV54" s="5"/>
     </row>
     <row r="55" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B55" s="163"/>
-      <c r="D55" s="160"/>
+      <c r="B55" s="177"/>
+      <c r="D55" s="170"/>
       <c r="E55" s="79" t="s">
         <v>102</v>
       </c>
@@ -8331,8 +8328,8 @@
       <c r="BV55" s="5"/>
     </row>
     <row r="56" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B56" s="163"/>
-      <c r="D56" s="160"/>
+      <c r="B56" s="177"/>
+      <c r="D56" s="170"/>
       <c r="E56" s="79" t="s">
         <v>102</v>
       </c>
@@ -8465,8 +8462,8 @@
       <c r="BV56" s="5"/>
     </row>
     <row r="57" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B57" s="163"/>
-      <c r="D57" s="160"/>
+      <c r="B57" s="177"/>
+      <c r="D57" s="170"/>
       <c r="E57" s="79" t="s">
         <v>102</v>
       </c>
@@ -8599,7 +8596,7 @@
       <c r="BV57" s="5"/>
     </row>
     <row r="58" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B58" s="163"/>
+      <c r="B58" s="177"/>
       <c r="D58" s="58"/>
       <c r="E58" s="82"/>
       <c r="F58" s="82"/>
@@ -8668,7 +8665,7 @@
       <c r="BV58" s="5"/>
     </row>
     <row r="59" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B59" s="163"/>
+      <c r="B59" s="177"/>
       <c r="D59" s="58"/>
       <c r="E59" s="82"/>
       <c r="F59" s="82"/>
@@ -8737,7 +8734,7 @@
       <c r="BV59" s="5"/>
     </row>
     <row r="60" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B60" s="163"/>
+      <c r="B60" s="177"/>
       <c r="D60" s="58"/>
       <c r="E60" s="82"/>
       <c r="F60" s="82"/>
@@ -8806,12 +8803,12 @@
       <c r="BV60" s="5"/>
     </row>
     <row r="61" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B61" s="163"/>
+      <c r="B61" s="177"/>
       <c r="D61" s="84"/>
       <c r="E61" s="82"/>
       <c r="F61" s="82"/>
       <c r="G61" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H61" s="1">
         <v>2022</v>
@@ -8902,8 +8899,8 @@
       </c>
     </row>
     <row r="62" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B62" s="163"/>
-      <c r="D62" s="158" t="s">
+      <c r="B62" s="177"/>
+      <c r="D62" s="168" t="s">
         <v>107</v>
       </c>
       <c r="E62" s="79" t="s">
@@ -9005,8 +9002,8 @@
       </c>
     </row>
     <row r="63" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B63" s="163"/>
-      <c r="D63" s="159"/>
+      <c r="B63" s="177"/>
+      <c r="D63" s="169"/>
       <c r="E63" s="82" t="s">
         <v>91</v>
       </c>
@@ -9106,8 +9103,8 @@
       </c>
     </row>
     <row r="64" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B64" s="163"/>
-      <c r="D64" s="159"/>
+      <c r="B64" s="177"/>
+      <c r="D64" s="169"/>
       <c r="E64" s="83" t="s">
         <v>91</v>
       </c>
@@ -9207,8 +9204,8 @@
       </c>
     </row>
     <row r="65" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B65" s="163"/>
-      <c r="D65" s="160"/>
+      <c r="B65" s="177"/>
+      <c r="D65" s="170"/>
       <c r="E65" s="79" t="s">
         <v>96</v>
       </c>
@@ -9308,8 +9305,8 @@
       </c>
     </row>
     <row r="66" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B66" s="163"/>
-      <c r="D66" s="160"/>
+      <c r="B66" s="177"/>
+      <c r="D66" s="170"/>
       <c r="E66" s="79" t="s">
         <v>96</v>
       </c>
@@ -9409,8 +9406,8 @@
       </c>
     </row>
     <row r="67" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B67" s="163"/>
-      <c r="D67" s="160"/>
+      <c r="B67" s="177"/>
+      <c r="D67" s="170"/>
       <c r="E67" s="79" t="s">
         <v>96</v>
       </c>
@@ -9510,8 +9507,8 @@
       </c>
     </row>
     <row r="68" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B68" s="163"/>
-      <c r="D68" s="160"/>
+      <c r="B68" s="177"/>
+      <c r="D68" s="170"/>
       <c r="E68" s="79" t="s">
         <v>98</v>
       </c>
@@ -9611,8 +9608,8 @@
       </c>
     </row>
     <row r="69" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B69" s="163"/>
-      <c r="D69" s="160"/>
+      <c r="B69" s="177"/>
+      <c r="D69" s="170"/>
       <c r="E69" s="79" t="s">
         <v>98</v>
       </c>
@@ -9712,8 +9709,8 @@
       </c>
     </row>
     <row r="70" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B70" s="163"/>
-      <c r="D70" s="160"/>
+      <c r="B70" s="177"/>
+      <c r="D70" s="170"/>
       <c r="E70" s="79" t="s">
         <v>98</v>
       </c>
@@ -9813,8 +9810,8 @@
       </c>
     </row>
     <row r="71" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B71" s="163"/>
-      <c r="D71" s="160"/>
+      <c r="B71" s="177"/>
+      <c r="D71" s="170"/>
       <c r="E71" s="79" t="s">
         <v>100</v>
       </c>
@@ -9947,8 +9944,8 @@
       <c r="BV71" s="5"/>
     </row>
     <row r="72" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B72" s="163"/>
-      <c r="D72" s="160"/>
+      <c r="B72" s="177"/>
+      <c r="D72" s="170"/>
       <c r="E72" s="79" t="s">
         <v>100</v>
       </c>
@@ -10081,8 +10078,8 @@
       <c r="BV72" s="5"/>
     </row>
     <row r="73" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B73" s="163"/>
-      <c r="D73" s="160"/>
+      <c r="B73" s="177"/>
+      <c r="D73" s="170"/>
       <c r="E73" s="79" t="s">
         <v>100</v>
       </c>
@@ -10215,8 +10212,8 @@
       <c r="BV73" s="5"/>
     </row>
     <row r="74" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B74" s="163"/>
-      <c r="D74" s="160"/>
+      <c r="B74" s="177"/>
+      <c r="D74" s="170"/>
       <c r="E74" s="79" t="s">
         <v>102</v>
       </c>
@@ -10349,8 +10346,8 @@
       <c r="BV74" s="5"/>
     </row>
     <row r="75" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B75" s="163"/>
-      <c r="D75" s="160"/>
+      <c r="B75" s="177"/>
+      <c r="D75" s="170"/>
       <c r="E75" s="79" t="s">
         <v>102</v>
       </c>
@@ -10483,8 +10480,8 @@
       <c r="BV75" s="5"/>
     </row>
     <row r="76" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B76" s="163"/>
-      <c r="D76" s="160"/>
+      <c r="B76" s="177"/>
+      <c r="D76" s="170"/>
       <c r="E76" s="79" t="s">
         <v>102</v>
       </c>
@@ -10617,18 +10614,18 @@
       <c r="BV76" s="5"/>
     </row>
     <row r="77" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B77" s="163"/>
+      <c r="B77" s="177"/>
       <c r="D77" s="84"/>
       <c r="E77" s="82"/>
       <c r="F77" s="82"/>
     </row>
     <row r="78" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B78" s="163"/>
+      <c r="B78" s="177"/>
       <c r="D78" s="40"/>
       <c r="E78" s="85"/>
       <c r="F78" s="85"/>
       <c r="G78" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H78" s="1">
         <v>2022</v>
@@ -10719,8 +10716,8 @@
       </c>
     </row>
     <row r="79" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B79" s="163"/>
-      <c r="D79" s="158" t="s">
+      <c r="B79" s="177"/>
+      <c r="D79" s="168" t="s">
         <v>108</v>
       </c>
       <c r="E79" s="79" t="s">
@@ -10822,8 +10819,8 @@
       <c r="AO79" s="1"/>
     </row>
     <row r="80" spans="2:74" x14ac:dyDescent="0.35">
-      <c r="B80" s="163"/>
-      <c r="D80" s="159"/>
+      <c r="B80" s="177"/>
+      <c r="D80" s="169"/>
       <c r="E80" s="82" t="s">
         <v>91</v>
       </c>
@@ -10923,8 +10920,8 @@
       <c r="AO80" s="1"/>
     </row>
     <row r="81" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B81" s="163"/>
-      <c r="D81" s="159"/>
+      <c r="B81" s="177"/>
+      <c r="D81" s="169"/>
       <c r="E81" s="83" t="s">
         <v>91</v>
       </c>
@@ -11024,8 +11021,8 @@
       <c r="AO81" s="1"/>
     </row>
     <row r="82" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B82" s="164"/>
-      <c r="D82" s="160"/>
+      <c r="B82" s="178"/>
+      <c r="D82" s="170"/>
       <c r="E82" s="79" t="s">
         <v>96</v>
       </c>
@@ -11124,8 +11121,8 @@
       </c>
     </row>
     <row r="83" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B83" s="164"/>
-      <c r="D83" s="160"/>
+      <c r="B83" s="178"/>
+      <c r="D83" s="170"/>
       <c r="E83" s="79" t="s">
         <v>96</v>
       </c>
@@ -11224,8 +11221,8 @@
       </c>
     </row>
     <row r="84" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B84" s="164"/>
-      <c r="D84" s="160"/>
+      <c r="B84" s="178"/>
+      <c r="D84" s="170"/>
       <c r="E84" s="79" t="s">
         <v>96</v>
       </c>
@@ -11326,8 +11323,8 @@
       <c r="AL84" s="5"/>
     </row>
     <row r="85" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B85" s="164"/>
-      <c r="D85" s="160"/>
+      <c r="B85" s="178"/>
+      <c r="D85" s="170"/>
       <c r="E85" s="79" t="s">
         <v>98</v>
       </c>
@@ -11428,8 +11425,8 @@
       <c r="AL85" s="5"/>
     </row>
     <row r="86" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B86" s="164"/>
-      <c r="D86" s="160"/>
+      <c r="B86" s="178"/>
+      <c r="D86" s="170"/>
       <c r="E86" s="79" t="s">
         <v>98</v>
       </c>
@@ -11530,8 +11527,8 @@
       <c r="AL86" s="5"/>
     </row>
     <row r="87" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B87" s="164"/>
-      <c r="D87" s="160"/>
+      <c r="B87" s="178"/>
+      <c r="D87" s="170"/>
       <c r="E87" s="79" t="s">
         <v>98</v>
       </c>
@@ -11632,8 +11629,8 @@
       <c r="AL87" s="5"/>
     </row>
     <row r="88" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B88" s="164"/>
-      <c r="D88" s="160"/>
+      <c r="B88" s="178"/>
+      <c r="D88" s="170"/>
       <c r="E88" s="79" t="s">
         <v>100</v>
       </c>
@@ -11734,8 +11731,8 @@
       <c r="AL88" s="5"/>
     </row>
     <row r="89" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B89" s="164"/>
-      <c r="D89" s="160"/>
+      <c r="B89" s="178"/>
+      <c r="D89" s="170"/>
       <c r="E89" s="79" t="s">
         <v>100</v>
       </c>
@@ -11836,8 +11833,8 @@
       <c r="AL89" s="5"/>
     </row>
     <row r="90" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B90" s="164"/>
-      <c r="D90" s="160"/>
+      <c r="B90" s="178"/>
+      <c r="D90" s="170"/>
       <c r="E90" s="79" t="s">
         <v>100</v>
       </c>
@@ -11938,8 +11935,8 @@
       <c r="AL90" s="5"/>
     </row>
     <row r="91" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B91" s="164"/>
-      <c r="D91" s="160"/>
+      <c r="B91" s="178"/>
+      <c r="D91" s="170"/>
       <c r="E91" s="79" t="s">
         <v>102</v>
       </c>
@@ -12040,8 +12037,8 @@
       <c r="AL91" s="5"/>
     </row>
     <row r="92" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B92" s="164"/>
-      <c r="D92" s="160"/>
+      <c r="B92" s="178"/>
+      <c r="D92" s="170"/>
       <c r="E92" s="79" t="s">
         <v>102</v>
       </c>
@@ -12142,8 +12139,8 @@
       <c r="AL92" s="5"/>
     </row>
     <row r="93" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B93" s="164"/>
-      <c r="D93" s="160"/>
+      <c r="B93" s="178"/>
+      <c r="D93" s="170"/>
       <c r="E93" s="79" t="s">
         <v>102</v>
       </c>
@@ -12244,12 +12241,12 @@
       <c r="AL93" s="5"/>
     </row>
     <row r="94" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B94" s="164"/>
+      <c r="B94" s="178"/>
     </row>
     <row r="95" spans="2:41" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B95" s="164"/>
+      <c r="B95" s="178"/>
       <c r="G95" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H95" s="1">
         <v>2022</v>
@@ -12340,8 +12337,8 @@
       </c>
     </row>
     <row r="96" spans="2:41" x14ac:dyDescent="0.35">
-      <c r="B96" s="164"/>
-      <c r="D96" s="158" t="s">
+      <c r="B96" s="178"/>
+      <c r="D96" s="168" t="s">
         <v>109</v>
       </c>
       <c r="E96" s="79" t="s">
@@ -12442,8 +12439,8 @@
       </c>
     </row>
     <row r="97" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B97" s="164"/>
-      <c r="D97" s="159"/>
+      <c r="B97" s="178"/>
+      <c r="D97" s="169"/>
       <c r="E97" s="82" t="s">
         <v>91</v>
       </c>
@@ -12542,8 +12539,8 @@
       </c>
     </row>
     <row r="98" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B98" s="164"/>
-      <c r="D98" s="159"/>
+      <c r="B98" s="178"/>
+      <c r="D98" s="169"/>
       <c r="E98" s="83" t="s">
         <v>91</v>
       </c>
@@ -12642,8 +12639,8 @@
       </c>
     </row>
     <row r="99" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B99" s="164"/>
-      <c r="D99" s="160"/>
+      <c r="B99" s="178"/>
+      <c r="D99" s="170"/>
       <c r="E99" s="79" t="s">
         <v>96</v>
       </c>
@@ -12742,8 +12739,8 @@
       </c>
     </row>
     <row r="100" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B100" s="164"/>
-      <c r="D100" s="160"/>
+      <c r="B100" s="178"/>
+      <c r="D100" s="170"/>
       <c r="E100" s="79" t="s">
         <v>96</v>
       </c>
@@ -12842,8 +12839,8 @@
       </c>
     </row>
     <row r="101" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B101" s="164"/>
-      <c r="D101" s="160"/>
+      <c r="B101" s="178"/>
+      <c r="D101" s="170"/>
       <c r="E101" s="79" t="s">
         <v>96</v>
       </c>
@@ -12942,8 +12939,8 @@
       </c>
     </row>
     <row r="102" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B102" s="164"/>
-      <c r="D102" s="160"/>
+      <c r="B102" s="178"/>
+      <c r="D102" s="170"/>
       <c r="E102" s="79" t="s">
         <v>98</v>
       </c>
@@ -13042,8 +13039,8 @@
       </c>
     </row>
     <row r="103" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B103" s="164"/>
-      <c r="D103" s="160"/>
+      <c r="B103" s="178"/>
+      <c r="D103" s="170"/>
       <c r="E103" s="79" t="s">
         <v>98</v>
       </c>
@@ -13142,8 +13139,8 @@
       </c>
     </row>
     <row r="104" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B104" s="164"/>
-      <c r="D104" s="160"/>
+      <c r="B104" s="178"/>
+      <c r="D104" s="170"/>
       <c r="E104" s="79" t="s">
         <v>98</v>
       </c>
@@ -13242,8 +13239,8 @@
       </c>
     </row>
     <row r="105" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B105" s="164"/>
-      <c r="D105" s="160"/>
+      <c r="B105" s="178"/>
+      <c r="D105" s="170"/>
       <c r="E105" s="79" t="s">
         <v>100</v>
       </c>
@@ -13342,8 +13339,8 @@
       </c>
     </row>
     <row r="106" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B106" s="164"/>
-      <c r="D106" s="160"/>
+      <c r="B106" s="178"/>
+      <c r="D106" s="170"/>
       <c r="E106" s="79" t="s">
         <v>100</v>
       </c>
@@ -13442,8 +13439,8 @@
       </c>
     </row>
     <row r="107" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B107" s="164"/>
-      <c r="D107" s="160"/>
+      <c r="B107" s="178"/>
+      <c r="D107" s="170"/>
       <c r="E107" s="79" t="s">
         <v>100</v>
       </c>
@@ -13542,8 +13539,8 @@
       </c>
     </row>
     <row r="108" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B108" s="164"/>
-      <c r="D108" s="160"/>
+      <c r="B108" s="178"/>
+      <c r="D108" s="170"/>
       <c r="E108" s="79" t="s">
         <v>102</v>
       </c>
@@ -13642,8 +13639,8 @@
       </c>
     </row>
     <row r="109" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B109" s="164"/>
-      <c r="D109" s="160"/>
+      <c r="B109" s="178"/>
+      <c r="D109" s="170"/>
       <c r="E109" s="79" t="s">
         <v>102</v>
       </c>
@@ -13742,8 +13739,8 @@
       </c>
     </row>
     <row r="110" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B110" s="164"/>
-      <c r="D110" s="160"/>
+      <c r="B110" s="178"/>
+      <c r="D110" s="170"/>
       <c r="E110" s="79" t="s">
         <v>102</v>
       </c>
@@ -13842,12 +13839,12 @@
       </c>
     </row>
     <row r="111" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B111" s="164"/>
+      <c r="B111" s="178"/>
     </row>
     <row r="112" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B112" s="164"/>
+      <c r="B112" s="178"/>
       <c r="G112" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H112" s="1">
         <v>2022</v>
@@ -13938,8 +13935,8 @@
       </c>
     </row>
     <row r="113" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B113" s="164"/>
-      <c r="D113" s="158" t="s">
+      <c r="B113" s="178"/>
+      <c r="D113" s="168" t="s">
         <v>110</v>
       </c>
       <c r="E113" s="79" t="s">
@@ -14041,8 +14038,8 @@
       </c>
     </row>
     <row r="114" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B114" s="164"/>
-      <c r="D114" s="159"/>
+      <c r="B114" s="178"/>
+      <c r="D114" s="169"/>
       <c r="E114" s="82" t="s">
         <v>91</v>
       </c>
@@ -14142,8 +14139,8 @@
       </c>
     </row>
     <row r="115" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B115" s="164"/>
-      <c r="D115" s="159"/>
+      <c r="B115" s="178"/>
+      <c r="D115" s="169"/>
       <c r="E115" s="83" t="s">
         <v>91</v>
       </c>
@@ -14243,8 +14240,8 @@
       </c>
     </row>
     <row r="116" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B116" s="164"/>
-      <c r="D116" s="160"/>
+      <c r="B116" s="178"/>
+      <c r="D116" s="170"/>
       <c r="E116" s="79" t="s">
         <v>96</v>
       </c>
@@ -14344,8 +14341,8 @@
       </c>
     </row>
     <row r="117" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B117" s="164"/>
-      <c r="D117" s="160"/>
+      <c r="B117" s="178"/>
+      <c r="D117" s="170"/>
       <c r="E117" s="79" t="s">
         <v>96</v>
       </c>
@@ -14445,8 +14442,8 @@
       </c>
     </row>
     <row r="118" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B118" s="164"/>
-      <c r="D118" s="160"/>
+      <c r="B118" s="178"/>
+      <c r="D118" s="170"/>
       <c r="E118" s="79" t="s">
         <v>96</v>
       </c>
@@ -14546,8 +14543,8 @@
       </c>
     </row>
     <row r="119" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B119" s="164"/>
-      <c r="D119" s="160"/>
+      <c r="B119" s="178"/>
+      <c r="D119" s="170"/>
       <c r="E119" s="79" t="s">
         <v>98</v>
       </c>
@@ -14647,8 +14644,8 @@
       </c>
     </row>
     <row r="120" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B120" s="164"/>
-      <c r="D120" s="160"/>
+      <c r="B120" s="178"/>
+      <c r="D120" s="170"/>
       <c r="E120" s="79" t="s">
         <v>98</v>
       </c>
@@ -14748,8 +14745,8 @@
       </c>
     </row>
     <row r="121" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B121" s="164"/>
-      <c r="D121" s="160"/>
+      <c r="B121" s="178"/>
+      <c r="D121" s="170"/>
       <c r="E121" s="79" t="s">
         <v>98</v>
       </c>
@@ -14849,8 +14846,8 @@
       </c>
     </row>
     <row r="122" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B122" s="164"/>
-      <c r="D122" s="160"/>
+      <c r="B122" s="178"/>
+      <c r="D122" s="170"/>
       <c r="E122" s="79" t="s">
         <v>100</v>
       </c>
@@ -14950,8 +14947,8 @@
       </c>
     </row>
     <row r="123" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B123" s="164"/>
-      <c r="D123" s="160"/>
+      <c r="B123" s="178"/>
+      <c r="D123" s="170"/>
       <c r="E123" s="79" t="s">
         <v>100</v>
       </c>
@@ -15051,8 +15048,8 @@
       </c>
     </row>
     <row r="124" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B124" s="164"/>
-      <c r="D124" s="160"/>
+      <c r="B124" s="178"/>
+      <c r="D124" s="170"/>
       <c r="E124" s="79" t="s">
         <v>100</v>
       </c>
@@ -15152,8 +15149,8 @@
       </c>
     </row>
     <row r="125" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B125" s="164"/>
-      <c r="D125" s="160"/>
+      <c r="B125" s="178"/>
+      <c r="D125" s="170"/>
       <c r="E125" s="79" t="s">
         <v>102</v>
       </c>
@@ -15253,8 +15250,8 @@
       </c>
     </row>
     <row r="126" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B126" s="164"/>
-      <c r="D126" s="160"/>
+      <c r="B126" s="178"/>
+      <c r="D126" s="170"/>
       <c r="E126" s="79" t="s">
         <v>102</v>
       </c>
@@ -15354,8 +15351,8 @@
       </c>
     </row>
     <row r="127" spans="2:36" x14ac:dyDescent="0.35">
-      <c r="B127" s="164"/>
-      <c r="D127" s="160"/>
+      <c r="B127" s="178"/>
+      <c r="D127" s="170"/>
       <c r="E127" s="79" t="s">
         <v>102</v>
       </c>
@@ -15458,23 +15455,23 @@
       <c r="B128" s="87"/>
     </row>
     <row r="129" spans="2:28" x14ac:dyDescent="0.35">
-      <c r="B129" s="162" t="s">
+      <c r="B129" s="171" t="s">
         <v>111</v>
       </c>
-      <c r="C129" s="161"/>
-      <c r="D129" s="161"/>
-      <c r="E129" s="161"/>
-      <c r="F129" s="161"/>
-      <c r="G129" s="161"/>
-      <c r="H129" s="161"/>
-      <c r="I129" s="161"/>
-      <c r="J129" s="161"/>
-      <c r="K129" s="161"/>
-      <c r="L129" s="161"/>
-      <c r="M129" s="161"/>
-      <c r="N129" s="161"/>
-      <c r="O129" s="161"/>
-      <c r="P129" s="161"/>
+      <c r="C129" s="145"/>
+      <c r="D129" s="145"/>
+      <c r="E129" s="145"/>
+      <c r="F129" s="145"/>
+      <c r="G129" s="145"/>
+      <c r="H129" s="145"/>
+      <c r="I129" s="145"/>
+      <c r="J129" s="145"/>
+      <c r="K129" s="145"/>
+      <c r="L129" s="145"/>
+      <c r="M129" s="145"/>
+      <c r="N129" s="145"/>
+      <c r="O129" s="145"/>
+      <c r="P129" s="145"/>
       <c r="Q129" s="50"/>
       <c r="R129" s="50"/>
       <c r="S129" s="50"/>
@@ -15509,21 +15506,21 @@
     </row>
     <row r="131" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B131" s="40"/>
-      <c r="C131" s="152" t="s">
+      <c r="C131" s="172" t="s">
         <v>112</v>
       </c>
-      <c r="D131" s="153"/>
-      <c r="E131" s="153"/>
-      <c r="F131" s="153"/>
-      <c r="G131" s="153"/>
-      <c r="H131" s="153"/>
-      <c r="I131" s="155" t="s">
+      <c r="D131" s="173"/>
+      <c r="E131" s="173"/>
+      <c r="F131" s="173"/>
+      <c r="G131" s="173"/>
+      <c r="H131" s="173"/>
+      <c r="I131" s="174" t="s">
         <v>113</v>
       </c>
-      <c r="J131" s="156"/>
-      <c r="K131" s="156"/>
-      <c r="L131" s="156"/>
-      <c r="M131" s="157"/>
+      <c r="J131" s="175"/>
+      <c r="K131" s="175"/>
+      <c r="L131" s="175"/>
+      <c r="M131" s="176"/>
       <c r="N131" s="89" t="s">
         <v>114</v>
       </c>
@@ -15541,14 +15538,14 @@
     </row>
     <row r="132" spans="2:28" ht="14.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B132" s="40"/>
-      <c r="C132" s="142" t="s">
+      <c r="C132" s="162" t="s">
         <v>116</v>
       </c>
-      <c r="D132" s="143"/>
-      <c r="E132" s="143"/>
-      <c r="F132" s="143"/>
-      <c r="G132" s="143"/>
-      <c r="H132" s="144"/>
+      <c r="D132" s="163"/>
+      <c r="E132" s="163"/>
+      <c r="F132" s="163"/>
+      <c r="G132" s="163"/>
+      <c r="H132" s="164"/>
       <c r="I132" t="s">
         <v>93</v>
       </c>
@@ -15559,14 +15556,14 @@
     </row>
     <row r="133" spans="2:28" ht="14.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B133" s="40"/>
-      <c r="C133" s="142" t="s">
+      <c r="C133" s="162" t="s">
         <v>117</v>
       </c>
-      <c r="D133" s="143"/>
-      <c r="E133" s="143"/>
-      <c r="F133" s="143"/>
-      <c r="G133" s="143"/>
-      <c r="H133" s="144"/>
+      <c r="D133" s="163"/>
+      <c r="E133" s="163"/>
+      <c r="F133" s="163"/>
+      <c r="G133" s="163"/>
+      <c r="H133" s="164"/>
       <c r="I133" s="100" t="s">
         <v>93</v>
       </c>
@@ -15589,21 +15586,21 @@
     </row>
     <row r="134" spans="2:28" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B134" s="40"/>
-      <c r="C134" s="142" t="s">
+      <c r="C134" s="162" t="s">
         <v>106</v>
       </c>
-      <c r="D134" s="143"/>
-      <c r="E134" s="143"/>
-      <c r="F134" s="143"/>
-      <c r="G134" s="143"/>
-      <c r="H134" s="144"/>
-      <c r="I134" s="148" t="s">
+      <c r="D134" s="163"/>
+      <c r="E134" s="163"/>
+      <c r="F134" s="163"/>
+      <c r="G134" s="163"/>
+      <c r="H134" s="164"/>
+      <c r="I134" s="165" t="s">
         <v>119</v>
       </c>
-      <c r="J134" s="149"/>
-      <c r="K134" s="149"/>
-      <c r="L134" s="149"/>
-      <c r="M134" s="150"/>
+      <c r="J134" s="166"/>
+      <c r="K134" s="166"/>
+      <c r="L134" s="166"/>
+      <c r="M134" s="167"/>
       <c r="N134" s="105"/>
       <c r="O134" s="105"/>
       <c r="P134" s="106"/>
@@ -15617,21 +15614,21 @@
     </row>
     <row r="135" spans="2:28" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B135" s="40"/>
-      <c r="C135" s="142" t="s">
+      <c r="C135" s="162" t="s">
         <v>120</v>
       </c>
-      <c r="D135" s="143"/>
-      <c r="E135" s="143"/>
-      <c r="F135" s="143"/>
-      <c r="G135" s="143"/>
-      <c r="H135" s="144"/>
-      <c r="I135" s="148" t="s">
+      <c r="D135" s="163"/>
+      <c r="E135" s="163"/>
+      <c r="F135" s="163"/>
+      <c r="G135" s="163"/>
+      <c r="H135" s="164"/>
+      <c r="I135" s="165" t="s">
         <v>121</v>
       </c>
-      <c r="J135" s="149"/>
-      <c r="K135" s="149"/>
-      <c r="L135" s="149"/>
-      <c r="M135" s="150"/>
+      <c r="J135" s="166"/>
+      <c r="K135" s="166"/>
+      <c r="L135" s="166"/>
+      <c r="M135" s="167"/>
       <c r="N135" s="105"/>
       <c r="O135" s="105"/>
       <c r="P135" s="106"/>
@@ -15645,14 +15642,14 @@
     </row>
     <row r="136" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B136" s="40"/>
-      <c r="C136" s="142" t="s">
+      <c r="C136" s="162" t="s">
         <v>122</v>
       </c>
-      <c r="D136" s="143"/>
-      <c r="E136" s="143"/>
-      <c r="F136" s="143"/>
-      <c r="G136" s="143"/>
-      <c r="H136" s="144"/>
+      <c r="D136" s="163"/>
+      <c r="E136" s="163"/>
+      <c r="F136" s="163"/>
+      <c r="G136" s="163"/>
+      <c r="H136" s="164"/>
       <c r="I136" s="108" t="s">
         <v>93</v>
       </c>
@@ -15673,14 +15670,14 @@
     </row>
     <row r="137" spans="2:28" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B137" s="40"/>
-      <c r="C137" s="145" t="s">
+      <c r="C137" s="179" t="s">
         <v>123</v>
       </c>
-      <c r="D137" s="146"/>
-      <c r="E137" s="146"/>
-      <c r="F137" s="146"/>
-      <c r="G137" s="146"/>
-      <c r="H137" s="147"/>
+      <c r="D137" s="180"/>
+      <c r="E137" s="180"/>
+      <c r="F137" s="180"/>
+      <c r="G137" s="180"/>
+      <c r="H137" s="181"/>
       <c r="I137" s="112" t="s">
         <v>93</v>
       </c>
@@ -15701,12 +15698,12 @@
     </row>
     <row r="138" spans="2:28" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B138" s="40"/>
-      <c r="C138" s="151"/>
-      <c r="D138" s="151"/>
-      <c r="E138" s="151"/>
-      <c r="F138" s="151"/>
-      <c r="G138" s="151"/>
-      <c r="H138" s="151"/>
+      <c r="C138" s="182"/>
+      <c r="D138" s="182"/>
+      <c r="E138" s="182"/>
+      <c r="F138" s="182"/>
+      <c r="G138" s="182"/>
+      <c r="H138" s="182"/>
       <c r="I138" s="116"/>
       <c r="J138" s="116"/>
       <c r="K138" s="116"/>
@@ -15725,21 +15722,21 @@
     </row>
     <row r="139" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B139" s="40"/>
-      <c r="C139" s="152" t="s">
+      <c r="C139" s="172" t="s">
         <v>124</v>
       </c>
-      <c r="D139" s="153"/>
-      <c r="E139" s="153"/>
-      <c r="F139" s="153"/>
-      <c r="G139" s="153"/>
-      <c r="H139" s="154"/>
-      <c r="I139" s="155" t="s">
+      <c r="D139" s="173"/>
+      <c r="E139" s="173"/>
+      <c r="F139" s="173"/>
+      <c r="G139" s="173"/>
+      <c r="H139" s="183"/>
+      <c r="I139" s="174" t="s">
         <v>113</v>
       </c>
-      <c r="J139" s="156"/>
-      <c r="K139" s="156"/>
-      <c r="L139" s="156"/>
-      <c r="M139" s="157"/>
+      <c r="J139" s="175"/>
+      <c r="K139" s="175"/>
+      <c r="L139" s="175"/>
+      <c r="M139" s="176"/>
       <c r="N139" s="89" t="s">
         <v>114</v>
       </c>
@@ -15757,14 +15754,14 @@
     </row>
     <row r="140" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B140" s="40"/>
-      <c r="C140" s="142" t="s">
+      <c r="C140" s="162" t="s">
         <v>117</v>
       </c>
-      <c r="D140" s="143"/>
-      <c r="E140" s="143"/>
-      <c r="F140" s="143"/>
-      <c r="G140" s="143"/>
-      <c r="H140" s="144"/>
+      <c r="D140" s="163"/>
+      <c r="E140" s="163"/>
+      <c r="F140" s="163"/>
+      <c r="G140" s="163"/>
+      <c r="H140" s="164"/>
       <c r="I140" s="100" t="s">
         <v>93</v>
       </c>
@@ -15848,14 +15845,14 @@
     </row>
     <row r="143" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B143" s="40"/>
-      <c r="C143" s="142" t="s">
+      <c r="C143" s="162" t="s">
         <v>120</v>
       </c>
-      <c r="D143" s="143"/>
-      <c r="E143" s="143"/>
-      <c r="F143" s="143"/>
-      <c r="G143" s="143"/>
-      <c r="H143" s="144"/>
+      <c r="D143" s="163"/>
+      <c r="E143" s="163"/>
+      <c r="F143" s="163"/>
+      <c r="G143" s="163"/>
+      <c r="H143" s="164"/>
       <c r="I143" s="122" t="s">
         <v>125</v>
       </c>
@@ -15876,14 +15873,14 @@
     </row>
     <row r="144" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B144" s="40"/>
-      <c r="C144" s="142" t="s">
+      <c r="C144" s="162" t="s">
         <v>122</v>
       </c>
-      <c r="D144" s="143"/>
-      <c r="E144" s="143"/>
-      <c r="F144" s="143"/>
-      <c r="G144" s="143"/>
-      <c r="H144" s="144"/>
+      <c r="D144" s="163"/>
+      <c r="E144" s="163"/>
+      <c r="F144" s="163"/>
+      <c r="G144" s="163"/>
+      <c r="H144" s="164"/>
       <c r="I144" s="122" t="s">
         <v>125</v>
       </c>
@@ -15904,14 +15901,14 @@
     </row>
     <row r="145" spans="2:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B145" s="40"/>
-      <c r="C145" s="145" t="s">
+      <c r="C145" s="179" t="s">
         <v>128</v>
       </c>
-      <c r="D145" s="146"/>
-      <c r="E145" s="146"/>
-      <c r="F145" s="146"/>
-      <c r="G145" s="146"/>
-      <c r="H145" s="147"/>
+      <c r="D145" s="180"/>
+      <c r="E145" s="180"/>
+      <c r="F145" s="180"/>
+      <c r="G145" s="180"/>
+      <c r="H145" s="181"/>
       <c r="I145" s="112" t="s">
         <v>93</v>
       </c>
@@ -16163,16 +16160,17 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="C7:Q7"/>
-    <mergeCell ref="B9:B36"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:L9"/>
-    <mergeCell ref="D11:L11"/>
-    <mergeCell ref="D12:L12"/>
-    <mergeCell ref="D13:L13"/>
-    <mergeCell ref="C15:P16"/>
+    <mergeCell ref="C140:H140"/>
+    <mergeCell ref="C143:H143"/>
+    <mergeCell ref="C144:H144"/>
+    <mergeCell ref="C145:H145"/>
+    <mergeCell ref="C135:H135"/>
+    <mergeCell ref="I135:M135"/>
+    <mergeCell ref="C136:H136"/>
+    <mergeCell ref="C137:H137"/>
+    <mergeCell ref="C138:H138"/>
+    <mergeCell ref="C139:H139"/>
+    <mergeCell ref="I139:M139"/>
     <mergeCell ref="C134:H134"/>
     <mergeCell ref="I134:M134"/>
     <mergeCell ref="D17:D27"/>
@@ -16189,17 +16187,16 @@
     <mergeCell ref="D79:D93"/>
     <mergeCell ref="D96:D110"/>
     <mergeCell ref="D113:D127"/>
-    <mergeCell ref="I135:M135"/>
-    <mergeCell ref="C136:H136"/>
-    <mergeCell ref="C137:H137"/>
-    <mergeCell ref="C138:H138"/>
-    <mergeCell ref="C139:H139"/>
-    <mergeCell ref="I139:M139"/>
-    <mergeCell ref="C140:H140"/>
-    <mergeCell ref="C143:H143"/>
-    <mergeCell ref="C144:H144"/>
-    <mergeCell ref="C145:H145"/>
-    <mergeCell ref="C135:H135"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="C7:Q7"/>
+    <mergeCell ref="B9:B36"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:L9"/>
+    <mergeCell ref="D11:L11"/>
+    <mergeCell ref="D12:L12"/>
+    <mergeCell ref="D13:L13"/>
+    <mergeCell ref="C15:P16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="M1" r:id="rId1" display="https://atb.nrel.gov/electricity/2022/utility-scale_battery_storage" xr:uid="{7816EC9A-0454-4087-A6E1-F971C99AA20E}"/>
@@ -17057,7 +17054,7 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B1">
         <v>2021</v>
@@ -17152,7 +17149,7 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B2">
         <v>272875</v>
@@ -17365,7 +17362,7 @@
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B5">
         <v>2021</v>
@@ -17460,7 +17457,7 @@
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B6">
         <v>253384</v>
@@ -17673,7 +17670,7 @@
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B9" t="s">
         <v>81</v>
@@ -17768,7 +17765,7 @@
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B10" t="s">
         <v>81</v>
@@ -17863,7 +17860,7 @@
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B12">
         <v>0.78500000000000003</v>
@@ -18460,43 +18457,173 @@
       <c r="A1" t="s">
         <v>130</v>
       </c>
-      <c r="B1" t="s">
-        <v>43</v>
+      <c r="B1">
+        <v>2024</v>
+      </c>
+      <c r="C1">
+        <v>2025</v>
+      </c>
+      <c r="D1">
+        <v>2026</v>
+      </c>
+      <c r="E1">
+        <v>2027</v>
+      </c>
+      <c r="F1">
+        <v>2028</v>
+      </c>
+      <c r="G1">
+        <v>2029</v>
+      </c>
+      <c r="H1">
+        <v>2030</v>
+      </c>
+      <c r="I1">
+        <v>2031</v>
+      </c>
+      <c r="J1">
+        <v>2032</v>
+      </c>
+      <c r="K1">
+        <v>2033</v>
+      </c>
+      <c r="L1">
+        <v>2034</v>
+      </c>
+      <c r="M1">
+        <v>2035</v>
+      </c>
+      <c r="N1">
+        <v>2036</v>
+      </c>
+      <c r="O1">
+        <v>2037</v>
+      </c>
+      <c r="P1">
+        <v>2038</v>
+      </c>
+      <c r="Q1">
+        <v>2039</v>
+      </c>
+      <c r="R1">
+        <v>2040</v>
+      </c>
+      <c r="S1">
+        <v>2041</v>
+      </c>
+      <c r="T1">
+        <v>2042</v>
+      </c>
+      <c r="U1">
+        <v>2043</v>
+      </c>
+      <c r="V1">
+        <v>2044</v>
+      </c>
+      <c r="W1">
+        <v>2045</v>
+      </c>
+      <c r="X1">
+        <v>2046</v>
+      </c>
+      <c r="Y1">
+        <v>2047</v>
+      </c>
+      <c r="Z1">
+        <v>2048</v>
+      </c>
+      <c r="AA1">
+        <v>2049</v>
+      </c>
+      <c r="AB1">
+        <v>2050</v>
       </c>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>131</v>
+        <v>43</v>
       </c>
       <c r="B2" s="36">
         <v>0.2</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="T2" s="5"/>
-      <c r="U2" s="5"/>
-      <c r="V2" s="5"/>
-      <c r="W2" s="5"/>
-      <c r="X2" s="5"/>
-      <c r="Y2" s="5"/>
-      <c r="Z2" s="5"/>
-      <c r="AA2" s="5"/>
-      <c r="AB2" s="5"/>
+      <c r="C2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="D2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="E2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="F2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="G2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="H2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="I2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="J2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="K2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="L2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="M2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="N2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="O2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="P2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="Q2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="R2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="S2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="T2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="U2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="V2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="W2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="X2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="Y2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="Z2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="AA2" s="36">
+        <v>0.2</v>
+      </c>
+      <c r="AB2" s="36">
+        <v>0.2</v>
+      </c>
       <c r="AC2" s="5"/>
       <c r="AD2" s="5"/>
       <c r="AE2" s="5"/>

</xml_diff>